<commit_message>
Add Deployment Validation sheet (S-21) to testing workbook
New sheet covers: pre-deployment checklist (8 items), step-by-step
deployment actions with timestamp log, 10 post-deployment smoke tests,
rollback plan with 5 steps, and deployment sign-off table.
Updated Cover index, Sign-Off summary, and Quick Reference card
to reflect all 21 testing categories (220+ total test cases).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013HebWtoa57fYQxkQjGjLgz
</commit_message>
<xml_diff>
--- a/PowerBI_Testing_Documentation.xlsx
+++ b/PowerBI_Testing_Documentation.xlsx
@@ -28,9 +28,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📤 S-18 Export &amp; Subscription Testing" sheetId="19" state="visible" r:id="rId19"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🔁 S-19 Regression Testing" sheetId="20" state="visible" r:id="rId20"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="✅ S-20 UAT Validation" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🐛 Defect Log" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🏁 Sign-Off" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="⚡ Quick Reference" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🚀 S-21 Deployment Validation" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🐛 Defect Log" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🏁 Sign-Off" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="⚡ Quick Reference" sheetId="25" state="visible" r:id="rId25"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -40,7 +41,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="26">
+  <fonts count="27">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -147,6 +148,12 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00C00000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
       <sz val="9"/>
     </font>
     <font>
@@ -224,6 +231,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00404040"/>
       </patternFill>
     </fill>
@@ -250,11 +262,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E2EFDA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -284,7 +291,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -367,11 +374,11 @@
     <xf numFmtId="0" fontId="17" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -382,10 +389,13 @@
     <xf numFmtId="0" fontId="12" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -394,37 +404,37 @@
     <xf numFmtId="0" fontId="16" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="26" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="26" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -792,7 +802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -853,7 +863,7 @@
       <c r="A8" s="1" t="n"/>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Comprehensive QA Framework  |  20 Testing Categories  |  Power BI Developers &amp; QA Teams</t>
+          <t>Comprehensive QA Framework  |  21 Testing Categories  |  Power BI Developers &amp; QA Teams</t>
         </is>
       </c>
       <c r="F8" s="1" t="n"/>
@@ -874,7 +884,7 @@
       <c r="A11" s="1" t="n"/>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Version 2.0  |  June 2026  |  QA / BI Centre of Excellence</t>
+          <t>Version 2.1  |  June 2026  |  QA / BI Centre of Excellence</t>
         </is>
       </c>
       <c r="F11" s="1" t="n"/>
@@ -1397,22 +1407,22 @@
     <row r="42" ht="18" customHeight="1">
       <c r="B42" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>21</t>
         </is>
       </c>
       <c r="C42" s="8" t="inlineStr">
         <is>
-          <t>🐛 Defect Log</t>
+          <t>🚀 Deployment Validation</t>
         </is>
       </c>
       <c r="D42" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>S-21</t>
         </is>
       </c>
       <c r="E42" s="8" t="inlineStr">
         <is>
-          <t>Defect tracking, severity, lifecycle</t>
+          <t>Pre/post deployment checks, smoke tests, rollback plan</t>
         </is>
       </c>
     </row>
@@ -1424,7 +1434,7 @@
       </c>
       <c r="C43" s="10" t="inlineStr">
         <is>
-          <t>🏁 Sign-Off</t>
+          <t>🐛 Defect Log</t>
         </is>
       </c>
       <c r="D43" s="10" t="inlineStr">
@@ -1434,7 +1444,7 @@
       </c>
       <c r="E43" s="10" t="inlineStr">
         <is>
-          <t>Final sign-off summary and approvals</t>
+          <t>Defect tracking, severity, lifecycle</t>
         </is>
       </c>
     </row>
@@ -1446,15 +1456,37 @@
       </c>
       <c r="C44" s="8" t="inlineStr">
         <is>
+          <t>🏁 Sign-Off</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>Final sign-off summary and approvals</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="18" customHeight="1">
+      <c r="B45" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C45" s="10" t="inlineStr">
+        <is>
           <t>⚡ Quick Reference</t>
         </is>
       </c>
-      <c r="D44" s="8" t="inlineStr">
+      <c r="D45" s="10" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E44" s="8" t="inlineStr">
+      <c r="E45" s="10" t="inlineStr">
         <is>
           <t>Quick check card for testers</t>
         </is>
@@ -8547,6 +8579,1127 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F53"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>🚀 S-21 DEPLOYMENT VALIDATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t>Validate the report is correctly deployed to production, smoke-tested, and a rollback plan is in place.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="8" customHeight="1"/>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>1. Pre-Deployment Checklist</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>Test ID</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>Validation Point</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="inlineStr">
+        <is>
+          <t>Steps / Action</t>
+        </is>
+      </c>
+      <c r="D5" s="15" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="F5" s="15" t="inlineStr">
+        <is>
+          <t>Pass / Fail</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>DV-01</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>All test phases signed off</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Confirm sign-off obtained for all 20 testing categories</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>All categories have ✅ sign-off</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr"/>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>☐ Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>DV-02</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>No open P1 or P2 defects</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>Review Defect Log — zero open Critical/High defects</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>Defect Log shows 0 open P1/P2</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr"/>
+      <c r="F7" s="19" t="inlineStr">
+        <is>
+          <t>☐ Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>DV-03</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Report version number confirmed</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Confirm .pbix file version and name match release spec</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Correct version labelled</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr"/>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>☐ Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>DV-04</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Deployment environment confirmed</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>Confirm target workspace (Prod) is correct</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>Correct workspace selected</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr"/>
+      <c r="F9" s="19" t="inlineStr">
+        <is>
+          <t>☐ Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>DV-05</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Backup of previous production report taken</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Download existing Prod .pbix as rollback backup</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>Backup .pbix saved and labelled</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr"/>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>☐ Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>DV-06</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Change log / release notes prepared</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>Confirm release notes document changes in this version</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>Release notes available</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr"/>
+      <c r="F11" s="19" t="inlineStr">
+        <is>
+          <t>☐ Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>DV-07</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Stakeholder deployment notification sent</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Send pre-deployment notification to impacted users</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Notification sent and acknowledged</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr"/>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>☐ Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>DV-08</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Deployment window approved</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>Confirm deployment scheduled in low-traffic window</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>Window approved by stakeholders</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="inlineStr"/>
+      <c r="F13" s="19" t="inlineStr">
+        <is>
+          <t>☐ Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="8" customHeight="1"/>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="14" t="inlineStr">
+        <is>
+          <t>2. Deployment Steps &amp; Verification</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>Performed By</t>
+        </is>
+      </c>
+      <c r="D16" s="15" t="inlineStr">
+        <is>
+          <t>Timestamp</t>
+        </is>
+      </c>
+      <c r="E16" s="15" t="inlineStr">
+        <is>
+          <t>Outcome</t>
+        </is>
+      </c>
+      <c r="F16" s="15" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Publish report from Power BI Desktop to Prod workspace</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr"/>
+      <c r="E17" s="8" t="inlineStr"/>
+      <c r="F17" s="8" t="inlineStr"/>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Verify report appears in Prod workspace</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr"/>
+      <c r="E18" s="10" t="inlineStr"/>
+      <c r="F18" s="10" t="inlineStr"/>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Bind dataset to Prod data source credentials</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr"/>
+      <c r="E19" s="8" t="inlineStr"/>
+      <c r="F19" s="8" t="inlineStr"/>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>Configure / verify scheduled refresh in Prod</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr"/>
+      <c r="E20" s="10" t="inlineStr"/>
+      <c r="F20" s="10" t="inlineStr"/>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Trigger manual data refresh and confirm success</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr"/>
+      <c r="E21" s="8" t="inlineStr"/>
+      <c r="F21" s="8" t="inlineStr"/>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>Verify RLS roles are applied in Prod workspace</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>Developer / QA</t>
+        </is>
+      </c>
+      <c r="D22" s="10" t="inlineStr"/>
+      <c r="E22" s="10" t="inlineStr"/>
+      <c r="F22" s="10" t="inlineStr"/>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>Publish Power BI App update (if applicable)</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr"/>
+      <c r="E23" s="8" t="inlineStr"/>
+      <c r="F23" s="8" t="inlineStr"/>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>Send deployment completion notification to stakeholders</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>Developer / PM</t>
+        </is>
+      </c>
+      <c r="D24" s="10" t="inlineStr"/>
+      <c r="E24" s="10" t="inlineStr"/>
+      <c r="F24" s="10" t="inlineStr"/>
+    </row>
+    <row r="25" ht="8" customHeight="1"/>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="14" t="inlineStr">
+        <is>
+          <t>3. Post-Deployment Smoke Tests</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="15" t="inlineStr">
+        <is>
+          <t>Test ID</t>
+        </is>
+      </c>
+      <c r="B27" s="15" t="inlineStr">
+        <is>
+          <t>Smoke Test</t>
+        </is>
+      </c>
+      <c r="C27" s="15" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="D27" s="15" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="E27" s="15" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="F27" s="15" t="inlineStr">
+        <is>
+          <t>Pass / Fail</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>SM-01</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>Report opens without error in Prod</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>Navigate to Prod workspace; open report</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>Report loads, no error banner</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr"/>
+      <c r="F28" s="18" t="inlineStr">
+        <is>
+          <t>☐ Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>SM-02</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>Data is current and refreshed</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>Check 'Last refreshed' timestamp in report</t>
+        </is>
+      </c>
+      <c r="D29" s="10" t="inlineStr">
+        <is>
+          <t>Timestamp shows latest refresh time</t>
+        </is>
+      </c>
+      <c r="E29" s="10" t="inlineStr"/>
+      <c r="F29" s="19" t="inlineStr">
+        <is>
+          <t>☐ Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>SM-03</t>
+        </is>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>Key KPIs show expected values</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>Compare key totals against pre-agreed baseline</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>Values within expected range</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr"/>
+      <c r="F30" s="18" t="inlineStr">
+        <is>
+          <t>☐ Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="10" t="inlineStr">
+        <is>
+          <t>SM-04</t>
+        </is>
+      </c>
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>All report pages accessible</t>
+        </is>
+      </c>
+      <c r="C31" s="10" t="inlineStr">
+        <is>
+          <t>Navigate to every page tab in the report</t>
+        </is>
+      </c>
+      <c r="D31" s="10" t="inlineStr">
+        <is>
+          <t>All pages load without error</t>
+        </is>
+      </c>
+      <c r="E31" s="10" t="inlineStr"/>
+      <c r="F31" s="19" t="inlineStr">
+        <is>
+          <t>☐ Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>SM-05</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>RLS restricts data correctly in Prod</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>Log in as RLS test user; verify data scope</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>Only permitted data visible</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr"/>
+      <c r="F32" s="18" t="inlineStr">
+        <is>
+          <t>☐ Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t>SM-06</t>
+        </is>
+      </c>
+      <c r="B33" s="10" t="inlineStr">
+        <is>
+          <t>Slicers and filters functional</t>
+        </is>
+      </c>
+      <c r="C33" s="10" t="inlineStr">
+        <is>
+          <t>Apply each slicer; verify visuals update</t>
+        </is>
+      </c>
+      <c r="D33" s="10" t="inlineStr">
+        <is>
+          <t>Slicers filter visuals correctly</t>
+        </is>
+      </c>
+      <c r="E33" s="10" t="inlineStr"/>
+      <c r="F33" s="19" t="inlineStr">
+        <is>
+          <t>☐ Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>SM-07</t>
+        </is>
+      </c>
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>Scheduled refresh enabled</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>Power BI Service → Dataset settings → Refresh</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>Refresh schedule is active</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr"/>
+      <c r="F34" s="18" t="inlineStr">
+        <is>
+          <t>☐ Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="10" t="inlineStr">
+        <is>
+          <t>SM-08</t>
+        </is>
+      </c>
+      <c r="B35" s="10" t="inlineStr">
+        <is>
+          <t>Power BI App shows updated content</t>
+        </is>
+      </c>
+      <c r="C35" s="10" t="inlineStr">
+        <is>
+          <t>Open App as end user; verify updated report visible</t>
+        </is>
+      </c>
+      <c r="D35" s="10" t="inlineStr">
+        <is>
+          <t>App reflects new version</t>
+        </is>
+      </c>
+      <c r="E35" s="10" t="inlineStr"/>
+      <c r="F35" s="19" t="inlineStr">
+        <is>
+          <t>☐ Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>SM-09</t>
+        </is>
+      </c>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>Export to PDF works in Prod</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>Export report to PDF; verify all pages</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>PDF generates without error</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr"/>
+      <c r="F36" s="18" t="inlineStr">
+        <is>
+          <t>☐ Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="10" t="inlineStr">
+        <is>
+          <t>SM-10</t>
+        </is>
+      </c>
+      <c r="B37" s="10" t="inlineStr">
+        <is>
+          <t>Email subscription delivers correctly</t>
+        </is>
+      </c>
+      <c r="C37" s="10" t="inlineStr">
+        <is>
+          <t>Trigger subscription; verify email received</t>
+        </is>
+      </c>
+      <c r="D37" s="10" t="inlineStr">
+        <is>
+          <t>Email delivered with correct content</t>
+        </is>
+      </c>
+      <c r="E37" s="10" t="inlineStr"/>
+      <c r="F37" s="19" t="inlineStr">
+        <is>
+          <t>☐ Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="8" customHeight="1"/>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="14" t="inlineStr">
+        <is>
+          <t>4. Rollback Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="30" t="inlineStr">
+        <is>
+          <t>Complete the rollback plan BEFORE deploying. If smoke tests fail, execute rollback immediately.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="15" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B41" s="15" t="inlineStr">
+        <is>
+          <t>Rollback Action</t>
+        </is>
+      </c>
+      <c r="C41" s="15" t="inlineStr">
+        <is>
+          <t>Performed By</t>
+        </is>
+      </c>
+      <c r="D41" s="15" t="inlineStr">
+        <is>
+          <t>Trigger Condition</t>
+        </is>
+      </c>
+      <c r="E41" s="15" t="inlineStr">
+        <is>
+          <t>Time Required</t>
+        </is>
+      </c>
+      <c r="F41" s="15" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="22" customHeight="1">
+      <c r="A42" s="8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B42" s="8" t="inlineStr">
+        <is>
+          <t>Re-publish previous backup .pbix to Prod workspace</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Any SM smoke test fails P1/P2</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>&lt; 15 min</t>
+        </is>
+      </c>
+      <c r="F42" s="8" t="inlineStr"/>
+    </row>
+    <row r="43" ht="22" customHeight="1">
+      <c r="A43" s="10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B43" s="10" t="inlineStr">
+        <is>
+          <t>Re-bind previous dataset credentials</t>
+        </is>
+      </c>
+      <c r="C43" s="10" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="D43" s="10" t="inlineStr">
+        <is>
+          <t>After re-publish</t>
+        </is>
+      </c>
+      <c r="E43" s="10" t="inlineStr">
+        <is>
+          <t>&lt; 5 min</t>
+        </is>
+      </c>
+      <c r="F43" s="10" t="inlineStr"/>
+    </row>
+    <row r="44" ht="22" customHeight="1">
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B44" s="8" t="inlineStr">
+        <is>
+          <t>Trigger manual refresh on restored version</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>After credential bind</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>&lt; Refresh SLA</t>
+        </is>
+      </c>
+      <c r="F44" s="8" t="inlineStr"/>
+    </row>
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="10" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B45" s="10" t="inlineStr">
+        <is>
+          <t>Verify data and RLS correct on rolled-back version</t>
+        </is>
+      </c>
+      <c r="C45" s="10" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="D45" s="10" t="inlineStr">
+        <is>
+          <t>After refresh</t>
+        </is>
+      </c>
+      <c r="E45" s="10" t="inlineStr">
+        <is>
+          <t>&lt; 15 min</t>
+        </is>
+      </c>
+      <c r="F45" s="10" t="inlineStr"/>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B46" s="8" t="inlineStr">
+        <is>
+          <t>Notify stakeholders of rollback and root cause</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>After rollback confirmed</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>Immediately</t>
+        </is>
+      </c>
+      <c r="F46" s="8" t="inlineStr"/>
+    </row>
+    <row r="47" ht="8" customHeight="1"/>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="14" t="inlineStr">
+        <is>
+          <t>5. Deployment Sign-Off</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="20" customHeight="1">
+      <c r="A49" s="15" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="B49" s="15" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C49" s="15" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="D49" s="15" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="E49" s="15" t="inlineStr">
+        <is>
+          <t>Signature</t>
+        </is>
+      </c>
+      <c r="F49" s="15" t="inlineStr">
+        <is>
+          <t>Comments</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="26" customHeight="1">
+      <c r="A50" s="21" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="B50" s="21" t="inlineStr"/>
+      <c r="C50" s="28" t="inlineStr">
+        <is>
+          <t>☐ Approved</t>
+        </is>
+      </c>
+      <c r="D50" s="21" t="inlineStr"/>
+      <c r="E50" s="21" t="inlineStr"/>
+      <c r="F50" s="21" t="inlineStr"/>
+    </row>
+    <row r="51" ht="26" customHeight="1">
+      <c r="A51" s="23" t="inlineStr">
+        <is>
+          <t>Lead Developer</t>
+        </is>
+      </c>
+      <c r="B51" s="23" t="inlineStr"/>
+      <c r="C51" s="29" t="inlineStr">
+        <is>
+          <t>☐ Approved</t>
+        </is>
+      </c>
+      <c r="D51" s="23" t="inlineStr"/>
+      <c r="E51" s="23" t="inlineStr"/>
+      <c r="F51" s="23" t="inlineStr"/>
+    </row>
+    <row r="52" ht="26" customHeight="1">
+      <c r="A52" s="21" t="inlineStr">
+        <is>
+          <t>Business Owner</t>
+        </is>
+      </c>
+      <c r="B52" s="21" t="inlineStr"/>
+      <c r="C52" s="28" t="inlineStr">
+        <is>
+          <t>☐ Approved</t>
+        </is>
+      </c>
+      <c r="D52" s="21" t="inlineStr"/>
+      <c r="E52" s="21" t="inlineStr"/>
+      <c r="F52" s="21" t="inlineStr"/>
+    </row>
+    <row r="53" ht="26" customHeight="1">
+      <c r="A53" s="23" t="inlineStr">
+        <is>
+          <t>Project Manager</t>
+        </is>
+      </c>
+      <c r="B53" s="23" t="inlineStr"/>
+      <c r="C53" s="29" t="inlineStr">
+        <is>
+          <t>☐ Approved</t>
+        </is>
+      </c>
+      <c r="D53" s="23" t="inlineStr"/>
+      <c r="E53" s="23" t="inlineStr"/>
+      <c r="F53" s="23" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A40:F40"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A48:F48"/>
+    <mergeCell ref="A26:F26"/>
+    <mergeCell ref="A39:F39"/>
+    <mergeCell ref="A15:F15"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:M37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -8581,14 +9734,14 @@
     </row>
     <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="30" t="inlineStr">
+      <c r="A4" s="31" t="inlineStr">
         <is>
           <t>Severity Reference</t>
         </is>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="31" t="inlineStr">
+      <c r="A5" s="32" t="inlineStr">
         <is>
           <t>P1 – Critical</t>
         </is>
@@ -8598,7 +9751,7 @@
           <t>Unusable / materially wrong data</t>
         </is>
       </c>
-      <c r="D5" s="32" t="inlineStr">
+      <c r="D5" s="33" t="inlineStr">
         <is>
           <t>P2 – High</t>
         </is>
@@ -8608,7 +9761,7 @@
           <t>Key functionality broken</t>
         </is>
       </c>
-      <c r="G5" s="33" t="inlineStr">
+      <c r="G5" s="34" t="inlineStr">
         <is>
           <t>P3 – Medium</t>
         </is>
@@ -8618,7 +9771,7 @@
           <t>Non-critical issue</t>
         </is>
       </c>
-      <c r="J5" s="34" t="inlineStr">
+      <c r="J5" s="35" t="inlineStr">
         <is>
           <t>P4 – Low</t>
         </is>
@@ -8710,7 +9863,7 @@
       <c r="J8" s="16" t="inlineStr"/>
       <c r="K8" s="16" t="inlineStr"/>
       <c r="L8" s="16" t="inlineStr"/>
-      <c r="M8" s="35" t="inlineStr">
+      <c r="M8" s="36" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -8729,7 +9882,7 @@
       <c r="J9" s="17" t="inlineStr"/>
       <c r="K9" s="17" t="inlineStr"/>
       <c r="L9" s="17" t="inlineStr"/>
-      <c r="M9" s="36" t="inlineStr">
+      <c r="M9" s="37" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -8748,7 +9901,7 @@
       <c r="J10" s="16" t="inlineStr"/>
       <c r="K10" s="16" t="inlineStr"/>
       <c r="L10" s="16" t="inlineStr"/>
-      <c r="M10" s="35" t="inlineStr">
+      <c r="M10" s="36" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -8767,7 +9920,7 @@
       <c r="J11" s="17" t="inlineStr"/>
       <c r="K11" s="17" t="inlineStr"/>
       <c r="L11" s="17" t="inlineStr"/>
-      <c r="M11" s="36" t="inlineStr">
+      <c r="M11" s="37" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -8786,7 +9939,7 @@
       <c r="J12" s="16" t="inlineStr"/>
       <c r="K12" s="16" t="inlineStr"/>
       <c r="L12" s="16" t="inlineStr"/>
-      <c r="M12" s="35" t="inlineStr">
+      <c r="M12" s="36" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -8805,7 +9958,7 @@
       <c r="J13" s="17" t="inlineStr"/>
       <c r="K13" s="17" t="inlineStr"/>
       <c r="L13" s="17" t="inlineStr"/>
-      <c r="M13" s="36" t="inlineStr">
+      <c r="M13" s="37" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -8824,7 +9977,7 @@
       <c r="J14" s="16" t="inlineStr"/>
       <c r="K14" s="16" t="inlineStr"/>
       <c r="L14" s="16" t="inlineStr"/>
-      <c r="M14" s="35" t="inlineStr">
+      <c r="M14" s="36" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -8843,7 +9996,7 @@
       <c r="J15" s="17" t="inlineStr"/>
       <c r="K15" s="17" t="inlineStr"/>
       <c r="L15" s="17" t="inlineStr"/>
-      <c r="M15" s="36" t="inlineStr">
+      <c r="M15" s="37" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -8862,7 +10015,7 @@
       <c r="J16" s="16" t="inlineStr"/>
       <c r="K16" s="16" t="inlineStr"/>
       <c r="L16" s="16" t="inlineStr"/>
-      <c r="M16" s="35" t="inlineStr">
+      <c r="M16" s="36" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -8881,7 +10034,7 @@
       <c r="J17" s="17" t="inlineStr"/>
       <c r="K17" s="17" t="inlineStr"/>
       <c r="L17" s="17" t="inlineStr"/>
-      <c r="M17" s="36" t="inlineStr">
+      <c r="M17" s="37" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -8900,7 +10053,7 @@
       <c r="J18" s="16" t="inlineStr"/>
       <c r="K18" s="16" t="inlineStr"/>
       <c r="L18" s="16" t="inlineStr"/>
-      <c r="M18" s="35" t="inlineStr">
+      <c r="M18" s="36" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -8919,7 +10072,7 @@
       <c r="J19" s="17" t="inlineStr"/>
       <c r="K19" s="17" t="inlineStr"/>
       <c r="L19" s="17" t="inlineStr"/>
-      <c r="M19" s="36" t="inlineStr">
+      <c r="M19" s="37" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -8938,7 +10091,7 @@
       <c r="J20" s="16" t="inlineStr"/>
       <c r="K20" s="16" t="inlineStr"/>
       <c r="L20" s="16" t="inlineStr"/>
-      <c r="M20" s="35" t="inlineStr">
+      <c r="M20" s="36" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -8957,7 +10110,7 @@
       <c r="J21" s="17" t="inlineStr"/>
       <c r="K21" s="17" t="inlineStr"/>
       <c r="L21" s="17" t="inlineStr"/>
-      <c r="M21" s="36" t="inlineStr">
+      <c r="M21" s="37" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -8976,7 +10129,7 @@
       <c r="J22" s="16" t="inlineStr"/>
       <c r="K22" s="16" t="inlineStr"/>
       <c r="L22" s="16" t="inlineStr"/>
-      <c r="M22" s="35" t="inlineStr">
+      <c r="M22" s="36" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -8995,7 +10148,7 @@
       <c r="J23" s="17" t="inlineStr"/>
       <c r="K23" s="17" t="inlineStr"/>
       <c r="L23" s="17" t="inlineStr"/>
-      <c r="M23" s="36" t="inlineStr">
+      <c r="M23" s="37" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -9014,7 +10167,7 @@
       <c r="J24" s="16" t="inlineStr"/>
       <c r="K24" s="16" t="inlineStr"/>
       <c r="L24" s="16" t="inlineStr"/>
-      <c r="M24" s="35" t="inlineStr">
+      <c r="M24" s="36" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -9033,7 +10186,7 @@
       <c r="J25" s="17" t="inlineStr"/>
       <c r="K25" s="17" t="inlineStr"/>
       <c r="L25" s="17" t="inlineStr"/>
-      <c r="M25" s="36" t="inlineStr">
+      <c r="M25" s="37" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -9052,7 +10205,7 @@
       <c r="J26" s="16" t="inlineStr"/>
       <c r="K26" s="16" t="inlineStr"/>
       <c r="L26" s="16" t="inlineStr"/>
-      <c r="M26" s="35" t="inlineStr">
+      <c r="M26" s="36" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -9071,7 +10224,7 @@
       <c r="J27" s="17" t="inlineStr"/>
       <c r="K27" s="17" t="inlineStr"/>
       <c r="L27" s="17" t="inlineStr"/>
-      <c r="M27" s="36" t="inlineStr">
+      <c r="M27" s="37" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -9090,7 +10243,7 @@
       <c r="J28" s="16" t="inlineStr"/>
       <c r="K28" s="16" t="inlineStr"/>
       <c r="L28" s="16" t="inlineStr"/>
-      <c r="M28" s="35" t="inlineStr">
+      <c r="M28" s="36" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -9109,7 +10262,7 @@
       <c r="J29" s="17" t="inlineStr"/>
       <c r="K29" s="17" t="inlineStr"/>
       <c r="L29" s="17" t="inlineStr"/>
-      <c r="M29" s="36" t="inlineStr">
+      <c r="M29" s="37" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -9128,7 +10281,7 @@
       <c r="J30" s="16" t="inlineStr"/>
       <c r="K30" s="16" t="inlineStr"/>
       <c r="L30" s="16" t="inlineStr"/>
-      <c r="M30" s="35" t="inlineStr">
+      <c r="M30" s="36" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -9147,7 +10300,7 @@
       <c r="J31" s="17" t="inlineStr"/>
       <c r="K31" s="17" t="inlineStr"/>
       <c r="L31" s="17" t="inlineStr"/>
-      <c r="M31" s="36" t="inlineStr">
+      <c r="M31" s="37" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -9166,7 +10319,7 @@
       <c r="J32" s="16" t="inlineStr"/>
       <c r="K32" s="16" t="inlineStr"/>
       <c r="L32" s="16" t="inlineStr"/>
-      <c r="M32" s="35" t="inlineStr">
+      <c r="M32" s="36" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -9185,7 +10338,7 @@
       <c r="J33" s="17" t="inlineStr"/>
       <c r="K33" s="17" t="inlineStr"/>
       <c r="L33" s="17" t="inlineStr"/>
-      <c r="M33" s="36" t="inlineStr">
+      <c r="M33" s="37" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -9204,7 +10357,7 @@
       <c r="J34" s="16" t="inlineStr"/>
       <c r="K34" s="16" t="inlineStr"/>
       <c r="L34" s="16" t="inlineStr"/>
-      <c r="M34" s="35" t="inlineStr">
+      <c r="M34" s="36" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -9223,7 +10376,7 @@
       <c r="J35" s="17" t="inlineStr"/>
       <c r="K35" s="17" t="inlineStr"/>
       <c r="L35" s="17" t="inlineStr"/>
-      <c r="M35" s="36" t="inlineStr">
+      <c r="M35" s="37" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -9242,7 +10395,7 @@
       <c r="J36" s="16" t="inlineStr"/>
       <c r="K36" s="16" t="inlineStr"/>
       <c r="L36" s="16" t="inlineStr"/>
-      <c r="M36" s="35" t="inlineStr">
+      <c r="M36" s="36" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -9261,7 +10414,7 @@
       <c r="J37" s="17" t="inlineStr"/>
       <c r="K37" s="17" t="inlineStr"/>
       <c r="L37" s="17" t="inlineStr"/>
-      <c r="M37" s="36" t="inlineStr">
+      <c r="M37" s="37" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -9281,13 +10434,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -9358,14 +10511,14 @@
           <t>01  Requirement Validation</t>
         </is>
       </c>
-      <c r="B6" s="37" t="inlineStr">
+      <c r="B6" s="38" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="C6" s="37" t="inlineStr"/>
-      <c r="D6" s="37" t="inlineStr"/>
-      <c r="E6" s="37" t="inlineStr"/>
+      <c r="C6" s="38" t="inlineStr"/>
+      <c r="D6" s="38" t="inlineStr"/>
+      <c r="E6" s="38" t="inlineStr"/>
       <c r="F6" s="28" t="inlineStr">
         <is>
           <t>☐ Pending</t>
@@ -9378,14 +10531,14 @@
           <t>02  Data Source Validation</t>
         </is>
       </c>
-      <c r="B7" s="38" t="inlineStr">
+      <c r="B7" s="39" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="C7" s="38" t="inlineStr"/>
-      <c r="D7" s="38" t="inlineStr"/>
-      <c r="E7" s="38" t="inlineStr"/>
+      <c r="C7" s="39" t="inlineStr"/>
+      <c r="D7" s="39" t="inlineStr"/>
+      <c r="E7" s="39" t="inlineStr"/>
       <c r="F7" s="29" t="inlineStr">
         <is>
           <t>☐ Pending</t>
@@ -9398,14 +10551,14 @@
           <t>03  Power Query (PQE) Testing</t>
         </is>
       </c>
-      <c r="B8" s="37" t="inlineStr">
+      <c r="B8" s="38" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="C8" s="37" t="inlineStr"/>
-      <c r="D8" s="37" t="inlineStr"/>
-      <c r="E8" s="37" t="inlineStr"/>
+      <c r="C8" s="38" t="inlineStr"/>
+      <c r="D8" s="38" t="inlineStr"/>
+      <c r="E8" s="38" t="inlineStr"/>
       <c r="F8" s="28" t="inlineStr">
         <is>
           <t>☐ Pending</t>
@@ -9418,14 +10571,14 @@
           <t>04  Data Validation</t>
         </is>
       </c>
-      <c r="B9" s="38" t="inlineStr">
+      <c r="B9" s="39" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="C9" s="38" t="inlineStr"/>
-      <c r="D9" s="38" t="inlineStr"/>
-      <c r="E9" s="38" t="inlineStr"/>
+      <c r="C9" s="39" t="inlineStr"/>
+      <c r="D9" s="39" t="inlineStr"/>
+      <c r="E9" s="39" t="inlineStr"/>
       <c r="F9" s="29" t="inlineStr">
         <is>
           <t>☐ Pending</t>
@@ -9438,14 +10591,14 @@
           <t>05  Data Model Testing</t>
         </is>
       </c>
-      <c r="B10" s="37" t="inlineStr">
+      <c r="B10" s="38" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="C10" s="37" t="inlineStr"/>
-      <c r="D10" s="37" t="inlineStr"/>
-      <c r="E10" s="37" t="inlineStr"/>
+      <c r="C10" s="38" t="inlineStr"/>
+      <c r="D10" s="38" t="inlineStr"/>
+      <c r="E10" s="38" t="inlineStr"/>
       <c r="F10" s="28" t="inlineStr">
         <is>
           <t>☐ Pending</t>
@@ -9458,14 +10611,14 @@
           <t>06  DAX Testing</t>
         </is>
       </c>
-      <c r="B11" s="38" t="inlineStr">
+      <c r="B11" s="39" t="inlineStr">
         <is>
           <t>17</t>
         </is>
       </c>
-      <c r="C11" s="38" t="inlineStr"/>
-      <c r="D11" s="38" t="inlineStr"/>
-      <c r="E11" s="38" t="inlineStr"/>
+      <c r="C11" s="39" t="inlineStr"/>
+      <c r="D11" s="39" t="inlineStr"/>
+      <c r="E11" s="39" t="inlineStr"/>
       <c r="F11" s="29" t="inlineStr">
         <is>
           <t>☐ Pending</t>
@@ -9478,14 +10631,14 @@
           <t>07  Functional Testing</t>
         </is>
       </c>
-      <c r="B12" s="37" t="inlineStr">
+      <c r="B12" s="38" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="C12" s="37" t="inlineStr"/>
-      <c r="D12" s="37" t="inlineStr"/>
-      <c r="E12" s="37" t="inlineStr"/>
+      <c r="C12" s="38" t="inlineStr"/>
+      <c r="D12" s="38" t="inlineStr"/>
+      <c r="E12" s="38" t="inlineStr"/>
       <c r="F12" s="28" t="inlineStr">
         <is>
           <t>☐ Pending</t>
@@ -9498,14 +10651,14 @@
           <t>08  Visual Validation</t>
         </is>
       </c>
-      <c r="B13" s="38" t="inlineStr">
+      <c r="B13" s="39" t="inlineStr">
         <is>
           <t>14</t>
         </is>
       </c>
-      <c r="C13" s="38" t="inlineStr"/>
-      <c r="D13" s="38" t="inlineStr"/>
-      <c r="E13" s="38" t="inlineStr"/>
+      <c r="C13" s="39" t="inlineStr"/>
+      <c r="D13" s="39" t="inlineStr"/>
+      <c r="E13" s="39" t="inlineStr"/>
       <c r="F13" s="29" t="inlineStr">
         <is>
           <t>☐ Pending</t>
@@ -9518,14 +10671,14 @@
           <t>09  Filter &amp; Slicer Testing</t>
         </is>
       </c>
-      <c r="B14" s="37" t="inlineStr">
+      <c r="B14" s="38" t="inlineStr">
         <is>
           <t>14</t>
         </is>
       </c>
-      <c r="C14" s="37" t="inlineStr"/>
-      <c r="D14" s="37" t="inlineStr"/>
-      <c r="E14" s="37" t="inlineStr"/>
+      <c r="C14" s="38" t="inlineStr"/>
+      <c r="D14" s="38" t="inlineStr"/>
+      <c r="E14" s="38" t="inlineStr"/>
       <c r="F14" s="28" t="inlineStr">
         <is>
           <t>☐ Pending</t>
@@ -9538,14 +10691,14 @@
           <t>10  Navigation Testing</t>
         </is>
       </c>
-      <c r="B15" s="38" t="inlineStr">
+      <c r="B15" s="39" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="C15" s="38" t="inlineStr"/>
-      <c r="D15" s="38" t="inlineStr"/>
-      <c r="E15" s="38" t="inlineStr"/>
+      <c r="C15" s="39" t="inlineStr"/>
+      <c r="D15" s="39" t="inlineStr"/>
+      <c r="E15" s="39" t="inlineStr"/>
       <c r="F15" s="29" t="inlineStr">
         <is>
           <t>☐ Pending</t>
@@ -9558,14 +10711,14 @@
           <t>11  UI/UX Testing</t>
         </is>
       </c>
-      <c r="B16" s="37" t="inlineStr">
+      <c r="B16" s="38" t="inlineStr">
         <is>
           <t>14</t>
         </is>
       </c>
-      <c r="C16" s="37" t="inlineStr"/>
-      <c r="D16" s="37" t="inlineStr"/>
-      <c r="E16" s="37" t="inlineStr"/>
+      <c r="C16" s="38" t="inlineStr"/>
+      <c r="D16" s="38" t="inlineStr"/>
+      <c r="E16" s="38" t="inlineStr"/>
       <c r="F16" s="28" t="inlineStr">
         <is>
           <t>☐ Pending</t>
@@ -9578,14 +10731,14 @@
           <t>12  Security Testing (RLS+OLS)</t>
         </is>
       </c>
-      <c r="B17" s="38" t="inlineStr">
+      <c r="B17" s="39" t="inlineStr">
         <is>
           <t>14</t>
         </is>
       </c>
-      <c r="C17" s="38" t="inlineStr"/>
-      <c r="D17" s="38" t="inlineStr"/>
-      <c r="E17" s="38" t="inlineStr"/>
+      <c r="C17" s="39" t="inlineStr"/>
+      <c r="D17" s="39" t="inlineStr"/>
+      <c r="E17" s="39" t="inlineStr"/>
       <c r="F17" s="29" t="inlineStr">
         <is>
           <t>☐ Pending</t>
@@ -9598,14 +10751,14 @@
           <t>13  Refresh Testing</t>
         </is>
       </c>
-      <c r="B18" s="37" t="inlineStr">
+      <c r="B18" s="38" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="C18" s="37" t="inlineStr"/>
-      <c r="D18" s="37" t="inlineStr"/>
-      <c r="E18" s="37" t="inlineStr"/>
+      <c r="C18" s="38" t="inlineStr"/>
+      <c r="D18" s="38" t="inlineStr"/>
+      <c r="E18" s="38" t="inlineStr"/>
       <c r="F18" s="28" t="inlineStr">
         <is>
           <t>☐ Pending</t>
@@ -9618,14 +10771,14 @@
           <t>14  Performance Testing</t>
         </is>
       </c>
-      <c r="B19" s="38" t="inlineStr">
+      <c r="B19" s="39" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="C19" s="38" t="inlineStr"/>
-      <c r="D19" s="38" t="inlineStr"/>
-      <c r="E19" s="38" t="inlineStr"/>
+      <c r="C19" s="39" t="inlineStr"/>
+      <c r="D19" s="39" t="inlineStr"/>
+      <c r="E19" s="39" t="inlineStr"/>
       <c r="F19" s="29" t="inlineStr">
         <is>
           <t>☐ Pending</t>
@@ -9638,14 +10791,14 @@
           <t>15  Accessibility Testing</t>
         </is>
       </c>
-      <c r="B20" s="37" t="inlineStr">
+      <c r="B20" s="38" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="C20" s="37" t="inlineStr"/>
-      <c r="D20" s="37" t="inlineStr"/>
-      <c r="E20" s="37" t="inlineStr"/>
+      <c r="C20" s="38" t="inlineStr"/>
+      <c r="D20" s="38" t="inlineStr"/>
+      <c r="E20" s="38" t="inlineStr"/>
       <c r="F20" s="28" t="inlineStr">
         <is>
           <t>☐ Pending</t>
@@ -9658,14 +10811,14 @@
           <t>16  Mobile Layout Testing</t>
         </is>
       </c>
-      <c r="B21" s="38" t="inlineStr">
+      <c r="B21" s="39" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="C21" s="38" t="inlineStr"/>
-      <c r="D21" s="38" t="inlineStr"/>
-      <c r="E21" s="38" t="inlineStr"/>
+      <c r="C21" s="39" t="inlineStr"/>
+      <c r="D21" s="39" t="inlineStr"/>
+      <c r="E21" s="39" t="inlineStr"/>
       <c r="F21" s="29" t="inlineStr">
         <is>
           <t>☐ Pending</t>
@@ -9678,14 +10831,14 @@
           <t>17  Power BI Service Sanity</t>
         </is>
       </c>
-      <c r="B22" s="37" t="inlineStr">
+      <c r="B22" s="38" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="C22" s="37" t="inlineStr"/>
-      <c r="D22" s="37" t="inlineStr"/>
-      <c r="E22" s="37" t="inlineStr"/>
+      <c r="C22" s="38" t="inlineStr"/>
+      <c r="D22" s="38" t="inlineStr"/>
+      <c r="E22" s="38" t="inlineStr"/>
       <c r="F22" s="28" t="inlineStr">
         <is>
           <t>☐ Pending</t>
@@ -9698,14 +10851,14 @@
           <t>18  Export &amp; Subscription</t>
         </is>
       </c>
-      <c r="B23" s="38" t="inlineStr">
+      <c r="B23" s="39" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="C23" s="38" t="inlineStr"/>
-      <c r="D23" s="38" t="inlineStr"/>
-      <c r="E23" s="38" t="inlineStr"/>
+      <c r="C23" s="39" t="inlineStr"/>
+      <c r="D23" s="39" t="inlineStr"/>
+      <c r="E23" s="39" t="inlineStr"/>
       <c r="F23" s="29" t="inlineStr">
         <is>
           <t>☐ Pending</t>
@@ -9718,14 +10871,14 @@
           <t>19  Regression Testing</t>
         </is>
       </c>
-      <c r="B24" s="37" t="inlineStr">
+      <c r="B24" s="38" t="inlineStr">
         <is>
           <t>Variable</t>
         </is>
       </c>
-      <c r="C24" s="37" t="inlineStr"/>
-      <c r="D24" s="37" t="inlineStr"/>
-      <c r="E24" s="37" t="inlineStr"/>
+      <c r="C24" s="38" t="inlineStr"/>
+      <c r="D24" s="38" t="inlineStr"/>
+      <c r="E24" s="38" t="inlineStr"/>
       <c r="F24" s="28" t="inlineStr">
         <is>
           <t>☐ Pending</t>
@@ -9738,14 +10891,14 @@
           <t>20  UAT Validation</t>
         </is>
       </c>
-      <c r="B25" s="38" t="inlineStr">
+      <c r="B25" s="39" t="inlineStr">
         <is>
           <t>Variable</t>
         </is>
       </c>
-      <c r="C25" s="38" t="inlineStr"/>
-      <c r="D25" s="38" t="inlineStr"/>
-      <c r="E25" s="38" t="inlineStr"/>
+      <c r="C25" s="39" t="inlineStr"/>
+      <c r="D25" s="39" t="inlineStr"/>
+      <c r="E25" s="39" t="inlineStr"/>
       <c r="F25" s="29" t="inlineStr">
         <is>
           <t>☐ Pending</t>
@@ -9753,168 +10906,188 @@
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="39" t="inlineStr">
+      <c r="A26" s="21" t="inlineStr">
+        <is>
+          <t>21  Deployment Validation</t>
+        </is>
+      </c>
+      <c r="B26" s="38" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="C26" s="38" t="inlineStr"/>
+      <c r="D26" s="38" t="inlineStr"/>
+      <c r="E26" s="38" t="inlineStr"/>
+      <c r="F26" s="28" t="inlineStr">
+        <is>
+          <t>☐ Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="40" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B26" s="40" t="inlineStr">
-        <is>
-          <t>206+</t>
-        </is>
-      </c>
-      <c r="C26" s="40" t="inlineStr"/>
-      <c r="D26" s="40" t="inlineStr"/>
-      <c r="E26" s="40" t="inlineStr"/>
-      <c r="F26" s="40" t="inlineStr"/>
-    </row>
-    <row r="28" ht="8" customHeight="1"/>
-    <row r="29" ht="22" customHeight="1">
-      <c r="A29" s="14" t="inlineStr">
+      <c r="B27" s="41" t="inlineStr">
+        <is>
+          <t>220+</t>
+        </is>
+      </c>
+      <c r="C27" s="41" t="inlineStr"/>
+      <c r="D27" s="41" t="inlineStr"/>
+      <c r="E27" s="41" t="inlineStr"/>
+      <c r="F27" s="41" t="inlineStr"/>
+    </row>
+    <row r="29" ht="8" customHeight="1"/>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="14" t="inlineStr">
         <is>
           <t>Approval Signatures</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="15" t="inlineStr">
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="15" t="inlineStr">
         <is>
           <t>Role</t>
         </is>
       </c>
-      <c r="B30" s="15" t="inlineStr">
+      <c r="B31" s="15" t="inlineStr">
         <is>
           <t>Full Name</t>
         </is>
       </c>
-      <c r="C30" s="15" t="inlineStr">
+      <c r="C31" s="15" t="inlineStr">
         <is>
           <t>Signature</t>
         </is>
       </c>
-      <c r="D30" s="15" t="inlineStr">
+      <c r="D31" s="15" t="inlineStr">
         <is>
           <t>Date Approved</t>
         </is>
       </c>
-      <c r="E30" s="15" t="inlineStr">
+      <c r="E31" s="15" t="inlineStr">
         <is>
           <t>Decision</t>
         </is>
       </c>
-      <c r="F30" s="15" t="inlineStr">
+      <c r="F31" s="15" t="inlineStr">
         <is>
           <t>Comments</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="28" customHeight="1">
-      <c r="A31" s="21" t="inlineStr">
+    <row r="32" ht="28" customHeight="1">
+      <c r="A32" s="21" t="inlineStr">
         <is>
           <t>QA Lead</t>
         </is>
       </c>
-      <c r="B31" s="21" t="inlineStr"/>
-      <c r="C31" s="21" t="inlineStr"/>
-      <c r="D31" s="21" t="inlineStr"/>
-      <c r="E31" s="28" t="inlineStr">
+      <c r="B32" s="21" t="inlineStr"/>
+      <c r="C32" s="21" t="inlineStr"/>
+      <c r="D32" s="21" t="inlineStr"/>
+      <c r="E32" s="28" t="inlineStr">
         <is>
           <t>☐ Approved</t>
         </is>
       </c>
-      <c r="F31" s="21" t="inlineStr"/>
-    </row>
-    <row r="32" ht="28" customHeight="1">
-      <c r="A32" s="23" t="inlineStr">
+      <c r="F32" s="21" t="inlineStr"/>
+    </row>
+    <row r="33" ht="28" customHeight="1">
+      <c r="A33" s="23" t="inlineStr">
         <is>
           <t>Lead Developer</t>
         </is>
       </c>
-      <c r="B32" s="23" t="inlineStr"/>
-      <c r="C32" s="23" t="inlineStr"/>
-      <c r="D32" s="23" t="inlineStr"/>
-      <c r="E32" s="29" t="inlineStr">
+      <c r="B33" s="23" t="inlineStr"/>
+      <c r="C33" s="23" t="inlineStr"/>
+      <c r="D33" s="23" t="inlineStr"/>
+      <c r="E33" s="29" t="inlineStr">
         <is>
           <t>☐ Approved</t>
         </is>
       </c>
-      <c r="F32" s="23" t="inlineStr"/>
-    </row>
-    <row r="33" ht="28" customHeight="1">
-      <c r="A33" s="21" t="inlineStr">
+      <c r="F33" s="23" t="inlineStr"/>
+    </row>
+    <row r="34" ht="28" customHeight="1">
+      <c r="A34" s="21" t="inlineStr">
         <is>
           <t>Business Owner</t>
         </is>
       </c>
-      <c r="B33" s="21" t="inlineStr"/>
-      <c r="C33" s="21" t="inlineStr"/>
-      <c r="D33" s="21" t="inlineStr"/>
-      <c r="E33" s="28" t="inlineStr">
+      <c r="B34" s="21" t="inlineStr"/>
+      <c r="C34" s="21" t="inlineStr"/>
+      <c r="D34" s="21" t="inlineStr"/>
+      <c r="E34" s="28" t="inlineStr">
         <is>
           <t>☐ Approved</t>
         </is>
       </c>
-      <c r="F33" s="21" t="inlineStr"/>
-    </row>
-    <row r="34" ht="28" customHeight="1">
-      <c r="A34" s="23" t="inlineStr">
+      <c r="F34" s="21" t="inlineStr"/>
+    </row>
+    <row r="35" ht="28" customHeight="1">
+      <c r="A35" s="23" t="inlineStr">
         <is>
           <t>Project Manager</t>
         </is>
       </c>
-      <c r="B34" s="23" t="inlineStr"/>
-      <c r="C34" s="23" t="inlineStr"/>
-      <c r="D34" s="23" t="inlineStr"/>
-      <c r="E34" s="29" t="inlineStr">
+      <c r="B35" s="23" t="inlineStr"/>
+      <c r="C35" s="23" t="inlineStr"/>
+      <c r="D35" s="23" t="inlineStr"/>
+      <c r="E35" s="29" t="inlineStr">
         <is>
           <t>☐ Approved</t>
         </is>
       </c>
-      <c r="F34" s="23" t="inlineStr"/>
-    </row>
-    <row r="35" ht="28" customHeight="1">
-      <c r="A35" s="21" t="inlineStr">
+      <c r="F35" s="23" t="inlineStr"/>
+    </row>
+    <row r="36" ht="28" customHeight="1">
+      <c r="A36" s="21" t="inlineStr">
         <is>
           <t>Data Architect</t>
         </is>
       </c>
-      <c r="B35" s="21" t="inlineStr"/>
-      <c r="C35" s="21" t="inlineStr"/>
-      <c r="D35" s="21" t="inlineStr"/>
-      <c r="E35" s="28" t="inlineStr">
+      <c r="B36" s="21" t="inlineStr"/>
+      <c r="C36" s="21" t="inlineStr"/>
+      <c r="D36" s="21" t="inlineStr"/>
+      <c r="E36" s="28" t="inlineStr">
         <is>
           <t>☐ Approved</t>
         </is>
       </c>
-      <c r="F35" s="21" t="inlineStr"/>
-    </row>
-    <row r="37" ht="8" customHeight="1"/>
-    <row r="38" ht="22" customHeight="1">
-      <c r="A38" s="30" t="inlineStr">
+      <c r="F36" s="21" t="inlineStr"/>
+    </row>
+    <row r="38" ht="8" customHeight="1"/>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="31" t="inlineStr">
         <is>
           <t>Go / No-Go Decision</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="26" customHeight="1">
-      <c r="A39" s="41" t="inlineStr">
+    <row r="40" ht="26" customHeight="1">
+      <c r="A40" s="42" t="inlineStr">
         <is>
           <t>✅  GO — Approved for deployment to production</t>
         </is>
       </c>
-      <c r="E39" s="42" t="inlineStr">
+      <c r="E40" s="43" t="inlineStr">
         <is>
           <t>☐  Select</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="26" customHeight="1">
-      <c r="A40" s="43" t="inlineStr">
+    <row r="41" ht="26" customHeight="1">
+      <c r="A41" s="44" t="inlineStr">
         <is>
           <t>🚫  NO-GO — Further testing / defect resolution required</t>
         </is>
       </c>
-      <c r="E40" s="42" t="inlineStr">
+      <c r="E41" s="43" t="inlineStr">
         <is>
           <t>☐  Select</t>
         </is>
@@ -9922,27 +11095,27 @@
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="A38:F38"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A40:D40"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A39:D39"/>
+    <mergeCell ref="E41:F41"/>
+    <mergeCell ref="E40:F40"/>
+    <mergeCell ref="A41:D41"/>
     <mergeCell ref="A4:F4"/>
-    <mergeCell ref="E40:F40"/>
-    <mergeCell ref="E39:F39"/>
-    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="A30:F30"/>
+    <mergeCell ref="A39:F39"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -9954,14 +11127,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="44" t="inlineStr">
+      <c r="A1" s="45" t="inlineStr">
         <is>
           <t>POWER BI TESTING — QUICK REFERENCE CARD</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="B2" s="45" t="inlineStr">
+      <c r="B2" s="46" t="inlineStr">
         <is>
           <t>All 20 testing categories at a glance. Use as a daily checklist during testing.</t>
         </is>
@@ -9969,154 +11142,154 @@
     </row>
     <row r="4" ht="8" customHeight="1"/>
     <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="46" t="inlineStr">
+      <c r="B5" s="47" t="inlineStr">
         <is>
           <t>REQUIREMENT VALIDATION</t>
         </is>
       </c>
-      <c r="C5" s="47" t="inlineStr">
+      <c r="C5" s="48" t="inlineStr">
         <is>
           <t>DATA SOURCE VALIDATION</t>
         </is>
       </c>
-      <c r="D5" s="46" t="inlineStr">
+      <c r="D5" s="47" t="inlineStr">
         <is>
           <t>POWER QUERY TESTING</t>
         </is>
       </c>
-      <c r="E5" s="47" t="inlineStr">
+      <c r="E5" s="48" t="inlineStr">
         <is>
           <t>DATA VALIDATION</t>
         </is>
       </c>
     </row>
     <row r="6" ht="17" customHeight="1">
-      <c r="B6" s="48" t="inlineStr">
+      <c r="B6" s="49" t="inlineStr">
         <is>
           <t>☑ All BRD KPIs present in report</t>
         </is>
       </c>
-      <c r="C6" s="48" t="inlineStr">
+      <c r="C6" s="49" t="inlineStr">
         <is>
           <t>☑ All connections succeed</t>
         </is>
       </c>
-      <c r="D6" s="48" t="inlineStr">
+      <c r="D6" s="49" t="inlineStr">
         <is>
           <t>☑ Source step loads correct table</t>
         </is>
       </c>
-      <c r="E6" s="48" t="inlineStr">
+      <c r="E6" s="49" t="inlineStr">
         <is>
           <t>☑ Row counts match source</t>
         </is>
       </c>
     </row>
     <row r="7" ht="17" customHeight="1">
-      <c r="B7" s="49" t="inlineStr">
+      <c r="B7" s="50" t="inlineStr">
         <is>
           <t>☑ Page structure matches wireframe</t>
         </is>
       </c>
-      <c r="C7" s="49" t="inlineStr">
+      <c r="C7" s="50" t="inlineStr">
         <is>
           <t>☑ Service account credentials used</t>
         </is>
       </c>
-      <c r="D7" s="49" t="inlineStr">
+      <c r="D7" s="50" t="inlineStr">
         <is>
           <t>☑ Column renaming correct</t>
         </is>
       </c>
-      <c r="E7" s="49" t="inlineStr">
+      <c r="E7" s="50" t="inlineStr">
         <is>
           <t>☑ Totals match SQL aggregations</t>
         </is>
       </c>
     </row>
     <row r="8" ht="17" customHeight="1">
-      <c r="B8" s="48" t="inlineStr">
+      <c r="B8" s="49" t="inlineStr">
         <is>
           <t>☑ Required filters/slicers present</t>
         </is>
       </c>
-      <c r="C8" s="48" t="inlineStr">
+      <c r="C8" s="49" t="inlineStr">
         <is>
           <t>☑ Gateway online and mapped</t>
         </is>
       </c>
-      <c r="D8" s="48" t="inlineStr">
+      <c r="D8" s="49" t="inlineStr">
         <is>
           <t>☑ Data types applied correctly</t>
         </is>
       </c>
-      <c r="E8" s="48" t="inlineStr">
+      <c r="E8" s="49" t="inlineStr">
         <is>
           <t>☑ Date MIN/MAX verified</t>
         </is>
       </c>
     </row>
     <row r="9" ht="17" customHeight="1">
-      <c r="B9" s="49" t="inlineStr">
+      <c r="B9" s="50" t="inlineStr">
         <is>
           <t>☑ Calculated metrics match BRD formulas</t>
         </is>
       </c>
-      <c r="C9" s="49" t="inlineStr">
+      <c r="C9" s="50" t="inlineStr">
         <is>
           <t>☑ Schema matches model expectations</t>
         </is>
       </c>
-      <c r="D9" s="49" t="inlineStr">
+      <c r="D9" s="50" t="inlineStr">
         <is>
           <t>☑ Filter steps remove correct rows</t>
         </is>
       </c>
-      <c r="E9" s="49" t="inlineStr">
+      <c r="E9" s="50" t="inlineStr">
         <is>
           <t>☑ Nulls handled correctly</t>
         </is>
       </c>
     </row>
     <row r="10" ht="17" customHeight="1">
-      <c r="B10" s="48" t="inlineStr">
+      <c r="B10" s="49" t="inlineStr">
         <is>
           <t>☑ Report titles match naming spec</t>
         </is>
       </c>
-      <c r="C10" s="48" t="inlineStr">
+      <c r="C10" s="49" t="inlineStr">
         <is>
           <t>☑ Correct environment connected</t>
         </is>
       </c>
-      <c r="D10" s="48" t="inlineStr">
+      <c r="D10" s="49" t="inlineStr">
         <is>
           <t>☑ Custom column formulas verified</t>
         </is>
       </c>
-      <c r="E10" s="48" t="inlineStr">
+      <c r="E10" s="49" t="inlineStr">
         <is>
           <t>☑ No unintended duplicates</t>
         </is>
       </c>
     </row>
     <row r="11" ht="17" customHeight="1">
-      <c r="B11" s="49" t="inlineStr">
+      <c r="B11" s="50" t="inlineStr">
         <is>
           <t>☑ Date range scope correct</t>
         </is>
       </c>
-      <c r="C11" s="49" t="inlineStr">
+      <c r="C11" s="50" t="inlineStr">
         <is>
           <t>☑ Row count matches at source</t>
         </is>
       </c>
-      <c r="D11" s="49" t="inlineStr">
+      <c r="D11" s="50" t="inlineStr">
         <is>
           <t>☑ No unhandled step errors</t>
         </is>
       </c>
-      <c r="E11" s="49" t="inlineStr">
+      <c r="E11" s="50" t="inlineStr">
         <is>
           <t>☑ Filter context changes values</t>
         </is>
@@ -10124,154 +11297,154 @@
     </row>
     <row r="13" ht="8" customHeight="1"/>
     <row r="14" ht="22" customHeight="1">
-      <c r="B14" s="46" t="inlineStr">
+      <c r="B14" s="47" t="inlineStr">
         <is>
           <t>DATA MODEL TESTING</t>
         </is>
       </c>
-      <c r="C14" s="47" t="inlineStr">
+      <c r="C14" s="48" t="inlineStr">
         <is>
           <t>DAX TESTING</t>
         </is>
       </c>
-      <c r="D14" s="46" t="inlineStr">
+      <c r="D14" s="47" t="inlineStr">
         <is>
           <t>FUNCTIONAL TESTING</t>
         </is>
       </c>
-      <c r="E14" s="47" t="inlineStr">
+      <c r="E14" s="48" t="inlineStr">
         <is>
           <t>VISUAL VALIDATION</t>
         </is>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
-      <c r="B15" s="48" t="inlineStr">
+      <c r="B15" s="49" t="inlineStr">
         <is>
           <t>☑ Star/snowflake schema verified</t>
         </is>
       </c>
-      <c r="C15" s="48" t="inlineStr">
+      <c r="C15" s="49" t="inlineStr">
         <is>
           <t>☑ Aggregations verified vs SQL</t>
         </is>
       </c>
-      <c r="D15" s="48" t="inlineStr">
+      <c r="D15" s="49" t="inlineStr">
         <is>
           <t>☑ Cross-filter works correctly</t>
         </is>
       </c>
-      <c r="E15" s="48" t="inlineStr">
+      <c r="E15" s="49" t="inlineStr">
         <is>
           <t>☑ Correct visual type used</t>
         </is>
       </c>
     </row>
     <row r="16" ht="17" customHeight="1">
-      <c r="B16" s="49" t="inlineStr">
+      <c r="B16" s="50" t="inlineStr">
         <is>
           <t>☑ All relationships defined</t>
         </is>
       </c>
-      <c r="C16" s="49" t="inlineStr">
+      <c r="C16" s="50" t="inlineStr">
         <is>
           <t>☑ YTD / MTD / YoY tested</t>
         </is>
       </c>
-      <c r="D16" s="49" t="inlineStr">
+      <c r="D16" s="50" t="inlineStr">
         <is>
           <t>☑ Drill-down all levels tested</t>
         </is>
       </c>
-      <c r="E16" s="49" t="inlineStr">
+      <c r="E16" s="50" t="inlineStr">
         <is>
           <t>☑ Axis labels correct</t>
         </is>
       </c>
     </row>
     <row r="17" ht="17" customHeight="1">
-      <c r="B17" s="48" t="inlineStr">
+      <c r="B17" s="49" t="inlineStr">
         <is>
           <t>☑ Cardinality correct</t>
         </is>
       </c>
-      <c r="C17" s="48" t="inlineStr">
+      <c r="C17" s="49" t="inlineStr">
         <is>
           <t>☑ CALCULATE context correct</t>
         </is>
       </c>
-      <c r="D17" s="48" t="inlineStr">
+      <c r="D17" s="49" t="inlineStr">
         <is>
           <t>☑ Drill-through context correct</t>
         </is>
       </c>
-      <c r="E17" s="48" t="inlineStr">
+      <c r="E17" s="49" t="inlineStr">
         <is>
           <t>☑ Totals/subtotals accurate</t>
         </is>
       </c>
     </row>
     <row r="18" ht="17" customHeight="1">
-      <c r="B18" s="49" t="inlineStr">
+      <c r="B18" s="50" t="inlineStr">
         <is>
           <t>☑ Date table marked and complete</t>
         </is>
       </c>
-      <c r="C18" s="49" t="inlineStr">
+      <c r="C18" s="50" t="inlineStr">
         <is>
           <t>☑ DIVIDE handles zero denom.</t>
         </is>
       </c>
-      <c r="D18" s="49" t="inlineStr">
+      <c r="D18" s="50" t="inlineStr">
         <is>
           <t>☑ Back button returns correctly</t>
         </is>
       </c>
-      <c r="E18" s="49" t="inlineStr">
+      <c r="E18" s="50" t="inlineStr">
         <is>
           <t>☑ Conditional formatting correct</t>
         </is>
       </c>
     </row>
     <row r="19" ht="17" customHeight="1">
-      <c r="B19" s="48" t="inlineStr">
+      <c r="B19" s="49" t="inlineStr">
         <is>
           <t>☑ No M:M relationships</t>
         </is>
       </c>
-      <c r="C19" s="48" t="inlineStr">
+      <c r="C19" s="49" t="inlineStr">
         <is>
           <t>☑ Blanks handled correctly</t>
         </is>
       </c>
-      <c r="D19" s="48" t="inlineStr">
+      <c r="D19" s="49" t="inlineStr">
         <is>
           <t>☑ Exports verified (PDF/PPT)</t>
         </is>
       </c>
-      <c r="E19" s="48" t="inlineStr">
+      <c r="E19" s="49" t="inlineStr">
         <is>
           <t>☑ Tooltips content correct</t>
         </is>
       </c>
     </row>
     <row r="20" ht="17" customHeight="1">
-      <c r="B20" s="49" t="inlineStr">
+      <c r="B20" s="50" t="inlineStr">
         <is>
           <t>☑ Unused columns removed</t>
         </is>
       </c>
-      <c r="C20" s="49" t="inlineStr">
+      <c r="C20" s="50" t="inlineStr">
         <is>
           <t>☑ Calculated columns spot-checked</t>
         </is>
       </c>
-      <c r="D20" s="49" t="inlineStr">
+      <c r="D20" s="50" t="inlineStr">
         <is>
           <t>☑ Q&amp;A returns correct results</t>
         </is>
       </c>
-      <c r="E20" s="49" t="inlineStr">
+      <c r="E20" s="50" t="inlineStr">
         <is>
           <t>☑ No truncated/overlapping labels</t>
         </is>
@@ -10279,154 +11452,154 @@
     </row>
     <row r="22" ht="8" customHeight="1"/>
     <row r="23" ht="22" customHeight="1">
-      <c r="B23" s="46" t="inlineStr">
+      <c r="B23" s="47" t="inlineStr">
         <is>
           <t>FILTER &amp; SLICER</t>
         </is>
       </c>
-      <c r="C23" s="47" t="inlineStr">
+      <c r="C23" s="48" t="inlineStr">
         <is>
           <t>NAVIGATION TESTING</t>
         </is>
       </c>
-      <c r="D23" s="46" t="inlineStr">
+      <c r="D23" s="47" t="inlineStr">
         <is>
           <t>UI/UX TESTING</t>
         </is>
       </c>
-      <c r="E23" s="47" t="inlineStr">
+      <c r="E23" s="48" t="inlineStr">
         <is>
           <t>SECURITY (RLS + OLS)</t>
         </is>
       </c>
     </row>
     <row r="24" ht="17" customHeight="1">
-      <c r="B24" s="48" t="inlineStr">
+      <c r="B24" s="49" t="inlineStr">
         <is>
           <t>☑ Single/multi-select correct</t>
         </is>
       </c>
-      <c r="C24" s="48" t="inlineStr">
+      <c r="C24" s="49" t="inlineStr">
         <is>
           <t>☑ All bookmarks restore state</t>
         </is>
       </c>
-      <c r="D24" s="48" t="inlineStr">
+      <c r="D24" s="49" t="inlineStr">
         <is>
           <t>☑ Visuals aligned to grid</t>
         </is>
       </c>
-      <c r="E24" s="48" t="inlineStr">
+      <c r="E24" s="49" t="inlineStr">
         <is>
           <t>☑ RLS tested per role</t>
         </is>
       </c>
     </row>
     <row r="25" ht="17" customHeight="1">
-      <c r="B25" s="49" t="inlineStr">
+      <c r="B25" s="50" t="inlineStr">
         <is>
           <t>☑ Date range slicer correct</t>
         </is>
       </c>
-      <c r="C25" s="49" t="inlineStr">
+      <c r="C25" s="50" t="inlineStr">
         <is>
           <t>☑ Drill-through filter context</t>
         </is>
       </c>
-      <c r="D25" s="49" t="inlineStr">
+      <c r="D25" s="50" t="inlineStr">
         <is>
           <t>☑ Fonts consistent throughout</t>
         </is>
       </c>
-      <c r="E25" s="49" t="inlineStr">
+      <c r="E25" s="50" t="inlineStr">
         <is>
           <t>☑ Totals reflect RLS scope only</t>
         </is>
       </c>
     </row>
     <row r="26" ht="17" customHeight="1">
-      <c r="B26" s="48" t="inlineStr">
+      <c r="B26" s="49" t="inlineStr">
         <is>
           <t>☑ Slicer sync across pages</t>
         </is>
       </c>
-      <c r="C26" s="48" t="inlineStr">
+      <c r="C26" s="49" t="inlineStr">
         <is>
           <t>☑ Back button works</t>
         </is>
       </c>
-      <c r="D26" s="48" t="inlineStr">
+      <c r="D26" s="49" t="inlineStr">
         <is>
           <t>☑ Colours match brand theme</t>
         </is>
       </c>
-      <c r="E26" s="48" t="inlineStr">
+      <c r="E26" s="49" t="inlineStr">
         <is>
           <t>☑ Dynamic RLS (USERNAME) correct</t>
         </is>
       </c>
     </row>
     <row r="27" ht="17" customHeight="1">
-      <c r="B27" s="49" t="inlineStr">
+      <c r="B27" s="50" t="inlineStr">
         <is>
           <t>☑ Default filter state correct</t>
         </is>
       </c>
-      <c r="C27" s="49" t="inlineStr">
+      <c r="C27" s="50" t="inlineStr">
         <is>
           <t>☑ Nav buttons link correctly</t>
         </is>
       </c>
-      <c r="D27" s="49" t="inlineStr">
+      <c r="D27" s="50" t="inlineStr">
         <is>
           <t>☑ Number formats consistent</t>
         </is>
       </c>
-      <c r="E27" s="49" t="inlineStr">
+      <c r="E27" s="50" t="inlineStr">
         <is>
           <t>☑ OLS hides correct tables/columns</t>
         </is>
       </c>
     </row>
     <row r="28" ht="17" customHeight="1">
-      <c r="B28" s="48" t="inlineStr">
+      <c r="B28" s="49" t="inlineStr">
         <is>
           <t>☑ Clear filter resets only that slicer</t>
         </is>
       </c>
-      <c r="C28" s="48" t="inlineStr">
+      <c r="C28" s="49" t="inlineStr">
         <is>
           <t>☑ Tooltip pages display</t>
         </is>
       </c>
-      <c r="D28" s="48" t="inlineStr">
+      <c r="D28" s="49" t="inlineStr">
         <is>
           <t>☑ Date formats consistent</t>
         </is>
       </c>
-      <c r="E28" s="48" t="inlineStr">
+      <c r="E28" s="49" t="inlineStr">
         <is>
           <t>☑ Workspace permissions verified</t>
         </is>
       </c>
     </row>
     <row r="29" ht="17" customHeight="1">
-      <c r="B29" s="49" t="inlineStr">
+      <c r="B29" s="50" t="inlineStr">
         <is>
           <t>☑ Report/page/visual filter scope</t>
         </is>
       </c>
-      <c r="C29" s="49" t="inlineStr">
+      <c r="C29" s="50" t="inlineStr">
         <is>
           <t>☑ External links open correctly</t>
         </is>
       </c>
-      <c r="D29" s="49" t="inlineStr">
+      <c r="D29" s="50" t="inlineStr">
         <is>
           <t>☑ Company logo applied</t>
         </is>
       </c>
-      <c r="E29" s="49" t="inlineStr">
+      <c r="E29" s="50" t="inlineStr">
         <is>
           <t>☑ PII masked / export restricted</t>
         </is>
@@ -10434,154 +11607,154 @@
     </row>
     <row r="31" ht="8" customHeight="1"/>
     <row r="32" ht="22" customHeight="1">
-      <c r="B32" s="46" t="inlineStr">
+      <c r="B32" s="47" t="inlineStr">
         <is>
           <t>REFRESH TESTING</t>
         </is>
       </c>
-      <c r="C32" s="47" t="inlineStr">
+      <c r="C32" s="48" t="inlineStr">
         <is>
           <t>PERFORMANCE TESTING</t>
         </is>
       </c>
-      <c r="D32" s="46" t="inlineStr">
+      <c r="D32" s="47" t="inlineStr">
         <is>
           <t>ACCESSIBILITY TESTING</t>
         </is>
       </c>
-      <c r="E32" s="47" t="inlineStr">
+      <c r="E32" s="48" t="inlineStr">
         <is>
           <t>MOBILE LAYOUT</t>
         </is>
       </c>
     </row>
     <row r="33" ht="17" customHeight="1">
-      <c r="B33" s="48" t="inlineStr">
+      <c r="B33" s="49" t="inlineStr">
         <is>
           <t>☑ Manual refresh succeeds</t>
         </is>
       </c>
-      <c r="C33" s="48" t="inlineStr">
+      <c r="C33" s="49" t="inlineStr">
         <is>
           <t>☑ Page load &lt; 5 seconds</t>
         </is>
       </c>
-      <c r="D33" s="48" t="inlineStr">
+      <c r="D33" s="49" t="inlineStr">
         <is>
           <t>☑ Alt text on all visuals</t>
         </is>
       </c>
-      <c r="E33" s="48" t="inlineStr">
+      <c r="E33" s="49" t="inlineStr">
         <is>
           <t>☑ Mobile layout configured</t>
         </is>
       </c>
     </row>
     <row r="34" ht="17" customHeight="1">
-      <c r="B34" s="49" t="inlineStr">
+      <c r="B34" s="50" t="inlineStr">
         <is>
           <t>☑ Scheduled refresh on time</t>
         </is>
       </c>
-      <c r="C34" s="49" t="inlineStr">
+      <c r="C34" s="50" t="inlineStr">
         <is>
           <t>☑ Visual render &lt; 500ms</t>
         </is>
       </c>
-      <c r="D34" s="49" t="inlineStr">
+      <c r="D34" s="50" t="inlineStr">
         <is>
           <t>☑ Tab order logical</t>
         </is>
       </c>
-      <c r="E34" s="49" t="inlineStr">
+      <c r="E34" s="50" t="inlineStr">
         <is>
           <t>☑ iOS app renders correctly</t>
         </is>
       </c>
     </row>
     <row r="35" ht="17" customHeight="1">
-      <c r="B35" s="48" t="inlineStr">
+      <c r="B35" s="49" t="inlineStr">
         <is>
           <t>☑ New data appears after refresh</t>
         </is>
       </c>
-      <c r="C35" s="48" t="inlineStr">
+      <c r="C35" s="49" t="inlineStr">
         <is>
           <t>☑ Slicer response &lt; 2 seconds</t>
         </is>
       </c>
-      <c r="D35" s="48" t="inlineStr">
+      <c r="D35" s="49" t="inlineStr">
         <is>
           <t>☑ Contrast ratio ≥4.5:1</t>
         </is>
       </c>
-      <c r="E35" s="48" t="inlineStr">
+      <c r="E35" s="49" t="inlineStr">
         <is>
           <t>☑ Android app renders correctly</t>
         </is>
       </c>
     </row>
     <row r="36" ht="17" customHeight="1">
-      <c r="B36" s="49" t="inlineStr">
+      <c r="B36" s="50" t="inlineStr">
         <is>
           <t>☑ Incremental partition correct</t>
         </is>
       </c>
-      <c r="C36" s="49" t="inlineStr">
+      <c r="C36" s="50" t="inlineStr">
         <is>
           <t>☑ Performance Analyzer run</t>
         </is>
       </c>
-      <c r="D36" s="49" t="inlineStr">
+      <c r="D36" s="50" t="inlineStr">
         <is>
           <t>☑ Info not by colour alone</t>
         </is>
       </c>
-      <c r="E36" s="49" t="inlineStr">
+      <c r="E36" s="50" t="inlineStr">
         <is>
           <t>☑ Portrait/landscape tested</t>
         </is>
       </c>
     </row>
     <row r="37" ht="17" customHeight="1">
-      <c r="B37" s="48" t="inlineStr">
+      <c r="B37" s="49" t="inlineStr">
         <is>
           <t>☑ Failure triggers alert email</t>
         </is>
       </c>
-      <c r="C37" s="48" t="inlineStr">
+      <c r="C37" s="49" t="inlineStr">
         <is>
           <t>☑ Slow visuals flagged (&gt;500ms)</t>
         </is>
       </c>
-      <c r="D37" s="48" t="inlineStr">
+      <c r="D37" s="49" t="inlineStr">
         <is>
           <t>☑ Screen reader describes visuals</t>
         </is>
       </c>
-      <c r="E37" s="48" t="inlineStr">
+      <c r="E37" s="49" t="inlineStr">
         <is>
           <t>☑ Touch interactions work</t>
         </is>
       </c>
     </row>
     <row r="38" ht="17" customHeight="1">
-      <c r="B38" s="49" t="inlineStr">
+      <c r="B38" s="50" t="inlineStr">
         <is>
           <t>☑ Refresh within SLA</t>
         </is>
       </c>
-      <c r="C38" s="49" t="inlineStr">
+      <c r="C38" s="50" t="inlineStr">
         <is>
           <t>☑ DirectQuery SLA met</t>
         </is>
       </c>
-      <c r="D38" s="49" t="inlineStr">
+      <c r="D38" s="50" t="inlineStr">
         <is>
           <t>☑ Colour-blind simulation done</t>
         </is>
       </c>
-      <c r="E38" s="49" t="inlineStr">
+      <c r="E38" s="50" t="inlineStr">
         <is>
           <t>☑ KPI cards legible on mobile</t>
         </is>
@@ -10589,156 +11762,220 @@
     </row>
     <row r="40" ht="8" customHeight="1"/>
     <row r="41" ht="22" customHeight="1">
-      <c r="B41" s="46" t="inlineStr">
+      <c r="B41" s="47" t="inlineStr">
         <is>
           <t>SERVICE SANITY</t>
         </is>
       </c>
-      <c r="C41" s="47" t="inlineStr">
+      <c r="C41" s="48" t="inlineStr">
         <is>
           <t>EXPORT &amp; SUBSCRIPTION</t>
         </is>
       </c>
-      <c r="D41" s="46" t="inlineStr">
+      <c r="D41" s="47" t="inlineStr">
         <is>
           <t>REGRESSION TESTING</t>
         </is>
       </c>
-      <c r="E41" s="47" t="inlineStr">
+      <c r="E41" s="48" t="inlineStr">
         <is>
           <t>UAT VALIDATION</t>
         </is>
       </c>
     </row>
     <row r="42" ht="17" customHeight="1">
-      <c r="B42" s="48" t="inlineStr">
+      <c r="B42" s="49" t="inlineStr">
         <is>
           <t>☑ Published to correct workspace</t>
         </is>
       </c>
-      <c r="C42" s="48" t="inlineStr">
+      <c r="C42" s="49" t="inlineStr">
         <is>
           <t>☑ PDF export all pages</t>
         </is>
       </c>
-      <c r="D42" s="48" t="inlineStr">
+      <c r="D42" s="49" t="inlineStr">
         <is>
           <t>☑ Change impact analysed</t>
         </is>
       </c>
-      <c r="E42" s="48" t="inlineStr">
+      <c r="E42" s="49" t="inlineStr">
         <is>
           <t>☑ UAT test cases distributed</t>
         </is>
       </c>
     </row>
     <row r="43" ht="17" customHeight="1">
-      <c r="B43" s="49" t="inlineStr">
+      <c r="B43" s="50" t="inlineStr">
         <is>
           <t>☑ App configured correctly</t>
         </is>
       </c>
-      <c r="C43" s="49" t="inlineStr">
+      <c r="C43" s="50" t="inlineStr">
         <is>
           <t>☑ PPT export correct</t>
         </is>
       </c>
-      <c r="D43" s="49" t="inlineStr">
+      <c r="D43" s="50" t="inlineStr">
         <is>
           <t>☑ Impacted areas re-tested</t>
         </is>
       </c>
-      <c r="E43" s="49" t="inlineStr">
+      <c r="E43" s="50" t="inlineStr">
         <is>
           <t>☑ Business users executed tests</t>
         </is>
       </c>
     </row>
     <row r="44" ht="17" customHeight="1">
-      <c r="B44" s="48" t="inlineStr">
+      <c r="B44" s="49" t="inlineStr">
         <is>
           <t>☑ Dashboard tiles current</t>
         </is>
       </c>
-      <c r="C44" s="48" t="inlineStr">
+      <c r="C44" s="49" t="inlineStr">
         <is>
           <t>☑ Underlying data export matches</t>
         </is>
       </c>
-      <c r="D44" s="48" t="inlineStr">
+      <c r="D44" s="49" t="inlineStr">
         <is>
           <t>☑ No new defects introduced</t>
         </is>
       </c>
-      <c r="E44" s="48" t="inlineStr">
+      <c r="E44" s="49" t="inlineStr">
         <is>
           <t>☑ All P1/P2 defects resolved</t>
         </is>
       </c>
     </row>
     <row r="45" ht="17" customHeight="1">
-      <c r="B45" s="49" t="inlineStr">
+      <c r="B45" s="50" t="inlineStr">
         <is>
           <t>☑ Embed code works</t>
         </is>
       </c>
-      <c r="C45" s="49" t="inlineStr">
+      <c r="C45" s="50" t="inlineStr">
         <is>
           <t>☑ Export disabled on sensitive reports</t>
         </is>
       </c>
-      <c r="D45" s="49" t="inlineStr">
+      <c r="D45" s="50" t="inlineStr">
         <is>
           <t>☑ Baseline results compared</t>
         </is>
       </c>
-      <c r="E45" s="49" t="inlineStr">
+      <c r="E45" s="50" t="inlineStr">
         <is>
           <t>☑ 90%+ test cases passed</t>
         </is>
       </c>
     </row>
     <row r="46" ht="17" customHeight="1">
-      <c r="B46" s="48" t="inlineStr">
+      <c r="B46" s="49" t="inlineStr">
         <is>
           <t>☑ Data alerts trigger</t>
         </is>
       </c>
-      <c r="C46" s="48" t="inlineStr">
+      <c r="C46" s="49" t="inlineStr">
         <is>
           <t>☑ Subscriptions deliver on time</t>
         </is>
       </c>
-      <c r="D46" s="48" t="inlineStr">
+      <c r="D46" s="49" t="inlineStr">
         <is>
           <t>☑ Regression log updated</t>
         </is>
       </c>
-      <c r="E46" s="48" t="inlineStr">
+      <c r="E46" s="49" t="inlineStr">
         <is>
           <t>☑ Data reconciled within ±0.01%</t>
         </is>
       </c>
     </row>
     <row r="47" ht="17" customHeight="1">
-      <c r="B47" s="49" t="inlineStr">
+      <c r="B47" s="50" t="inlineStr">
         <is>
           <t>☑ Shared links work for recipients</t>
         </is>
       </c>
-      <c r="C47" s="49" t="inlineStr">
+      <c r="C47" s="50" t="inlineStr">
         <is>
           <t>☑ Subscription respects RLS</t>
         </is>
       </c>
-      <c r="D47" s="49" t="inlineStr">
+      <c r="D47" s="50" t="inlineStr">
         <is>
           <t>☑ Sign-off after regression</t>
         </is>
       </c>
-      <c r="E47" s="49" t="inlineStr">
+      <c r="E47" s="50" t="inlineStr">
         <is>
           <t>☑ Business Owner signed off</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="8" customHeight="1"/>
+    <row r="50" ht="22" customHeight="1">
+      <c r="B50" s="47" t="inlineStr">
+        <is>
+          <t>DEPLOYMENT VALIDATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="17" customHeight="1">
+      <c r="B51" s="49" t="inlineStr">
+        <is>
+          <t>☑ All 21 test phases signed off</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="17" customHeight="1">
+      <c r="B52" s="50" t="inlineStr">
+        <is>
+          <t>☑ No open P1/P2 defects</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="17" customHeight="1">
+      <c r="B53" s="49" t="inlineStr">
+        <is>
+          <t>☑ Prod backup taken (rollback ready)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="17" customHeight="1">
+      <c r="B54" s="50" t="inlineStr">
+        <is>
+          <t>☑ Release notes prepared</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="17" customHeight="1">
+      <c r="B55" s="49" t="inlineStr">
+        <is>
+          <t>☑ Smoke tests passed in Prod</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="17" customHeight="1">
+      <c r="B56" s="50" t="inlineStr">
+        <is>
+          <t>☑ RLS verified in Prod environment</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="17" customHeight="1">
+      <c r="B57" s="49" t="inlineStr">
+        <is>
+          <t>☑ Scheduled refresh confirmed active</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="17" customHeight="1">
+      <c r="B58" s="50" t="inlineStr">
+        <is>
+          <t>☑ Stakeholders notified</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reorder sheets to match standard Power BI testing lifecycle sequence
New order: Requirements → Data Sources → Power Query → Data Validation →
Data Model → DAX → Functional → Filter & Slicer → Navigation → Visual
Validation → UI/UX → Security → Refresh → Performance → Accessibility →
Mobile → Service Sanity → Export & Subscription → Regression → UAT →
Deployment Validation.

Moved Filter & Slicer (was pos 10) to pos 8, Navigation (pos 11) to pos 9,
Visual Validation (pos 9) to pos 10. Updated Cover index and Sign-Off
category list to reflect lifecycle sequence. Added flow logic banner to Cover.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013HebWtoa57fYQxkQjGjLgz
</commit_message>
<xml_diff>
--- a/PowerBI_Testing_Documentation.xlsx
+++ b/PowerBI_Testing_Documentation.xlsx
@@ -15,9 +15,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🏗 S-05 Data Model Testing" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🔢 S-06 DAX Testing" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🖱 S-07 Functional Testing" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="👁 S-08 Visual Validation" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🔽 S-09 Filter &amp; Slicer Testing" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🧭 S-10 Navigation Testing" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🔽 S-09 Filter &amp; Slicer Testing" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🧭 S-10 Navigation Testing" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="👁 S-08 Visual Validation" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🎨 S-11 UI-UX Testing" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🔒 S-12 Security Testing" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🔄 S-13 Refresh Testing" sheetId="14" state="visible" r:id="rId14"/>
@@ -41,7 +41,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="27">
+  <fonts count="28">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -196,6 +196,12 @@
       <color rgb="00375623"/>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00BDD7EE"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="14">
     <fill>
@@ -265,7 +271,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -287,11 +293,56 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -437,6 +488,12 @@
     <xf numFmtId="0" fontId="26" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -802,7 +859,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -965,6 +1022,7 @@
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="51" t="n"/>
       <c r="B22" s="8" t="inlineStr">
         <is>
           <t>01</t>
@@ -972,7 +1030,7 @@
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>📝 Requirement Validation</t>
+          <t>📝 S-01 Requirement Validation</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr">
@@ -985,8 +1043,10 @@
           <t>Validate report against business requirements &amp; BRD</t>
         </is>
       </c>
+      <c r="F22" s="51" t="n"/>
     </row>
     <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="51" t="n"/>
       <c r="B23" s="10" t="inlineStr">
         <is>
           <t>02</t>
@@ -994,7 +1054,7 @@
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>🗄 Data Source Validation</t>
+          <t>🗄 S-02 Data Source Validation</t>
         </is>
       </c>
       <c r="D23" s="10" t="inlineStr">
@@ -1007,8 +1067,10 @@
           <t>Verify source connections, credentials, gateway, schema</t>
         </is>
       </c>
+      <c r="F23" s="51" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="51" t="n"/>
       <c r="B24" s="8" t="inlineStr">
         <is>
           <t>03</t>
@@ -1016,7 +1078,7 @@
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>🔧 Power Query (PQE)</t>
+          <t>🔧 S-03 Power Query (PQE) Testing</t>
         </is>
       </c>
       <c r="D24" s="8" t="inlineStr">
@@ -1029,8 +1091,10 @@
           <t>Test M-code transformations, steps, and data shaping</t>
         </is>
       </c>
+      <c r="F24" s="51" t="n"/>
     </row>
     <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="51" t="n"/>
       <c r="B25" s="10" t="inlineStr">
         <is>
           <t>04</t>
@@ -1038,7 +1102,7 @@
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>📊 Data Validation</t>
+          <t>📊 S-04 Data Validation</t>
         </is>
       </c>
       <c r="D25" s="10" t="inlineStr">
@@ -1051,8 +1115,10 @@
           <t>Source-to-report reconciliation and data accuracy</t>
         </is>
       </c>
+      <c r="F25" s="51" t="n"/>
     </row>
     <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="51" t="n"/>
       <c r="B26" s="8" t="inlineStr">
         <is>
           <t>05</t>
@@ -1060,7 +1126,7 @@
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>🏗 Data Model Testing</t>
+          <t>🏗 S-05 Data Model Testing</t>
         </is>
       </c>
       <c r="D26" s="8" t="inlineStr">
@@ -1073,8 +1139,10 @@
           <t>Relationships, cardinality, schema, and table validation</t>
         </is>
       </c>
+      <c r="F26" s="51" t="n"/>
     </row>
     <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="51" t="n"/>
       <c r="B27" s="10" t="inlineStr">
         <is>
           <t>06</t>
@@ -1082,7 +1150,7 @@
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>🔢 DAX Testing</t>
+          <t>🔢 S-06 DAX Testing</t>
         </is>
       </c>
       <c r="D27" s="10" t="inlineStr">
@@ -1095,8 +1163,10 @@
           <t>Measures, calculated columns, time intelligence, context</t>
         </is>
       </c>
+      <c r="F27" s="51" t="n"/>
     </row>
     <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="51" t="n"/>
       <c r="B28" s="8" t="inlineStr">
         <is>
           <t>07</t>
@@ -1104,7 +1174,7 @@
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>🖱 Functional Testing</t>
+          <t>🖱 S-07 Functional Testing</t>
         </is>
       </c>
       <c r="D28" s="8" t="inlineStr">
@@ -1114,11 +1184,13 @@
       </c>
       <c r="E28" s="8" t="inlineStr">
         <is>
-          <t>Slicers, cross-filter, drill-down, export, interactions</t>
-        </is>
-      </c>
+          <t>Cross-filters, drill-down, interactions, export</t>
+        </is>
+      </c>
+      <c r="F28" s="51" t="n"/>
     </row>
     <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="51" t="n"/>
       <c r="B29" s="10" t="inlineStr">
         <is>
           <t>08</t>
@@ -1126,65 +1198,71 @@
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>👁 Visual Validation</t>
+          <t>🔽 S-09 Filter &amp; Slicer Testing</t>
         </is>
       </c>
       <c r="D29" s="10" t="inlineStr">
         <is>
+          <t>S-09</t>
+        </is>
+      </c>
+      <c r="E29" s="10" t="inlineStr">
+        <is>
+          <t>All filter and slicer types, sync, and default states</t>
+        </is>
+      </c>
+      <c r="F29" s="51" t="n"/>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="51" t="n"/>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>🧭 S-10 Navigation Testing</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>S-10</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>Bookmarks, drill-through, buttons, page links</t>
+        </is>
+      </c>
+      <c r="F30" s="51" t="n"/>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="51" t="n"/>
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C31" s="10" t="inlineStr">
+        <is>
+          <t>👁 S-08 Visual Validation</t>
+        </is>
+      </c>
+      <c r="D31" s="10" t="inlineStr">
+        <is>
           <t>S-08</t>
         </is>
       </c>
-      <c r="E29" s="10" t="inlineStr">
+      <c r="E31" s="10" t="inlineStr">
         <is>
           <t>Chart types, formatting, tooltips, totals, axis labels</t>
         </is>
       </c>
-    </row>
-    <row r="30" ht="18" customHeight="1">
-      <c r="B30" s="8" t="inlineStr">
-        <is>
-          <t>09</t>
-        </is>
-      </c>
-      <c r="C30" s="9" t="inlineStr">
-        <is>
-          <t>🔽 Filter &amp; Slicer</t>
-        </is>
-      </c>
-      <c r="D30" s="8" t="inlineStr">
-        <is>
-          <t>S-09</t>
-        </is>
-      </c>
-      <c r="E30" s="8" t="inlineStr">
-        <is>
-          <t>All filter and slicer types, sync, default states</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="18" customHeight="1">
-      <c r="B31" s="10" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="C31" s="10" t="inlineStr">
-        <is>
-          <t>🧭 Navigation Testing</t>
-        </is>
-      </c>
-      <c r="D31" s="10" t="inlineStr">
-        <is>
-          <t>S-10</t>
-        </is>
-      </c>
-      <c r="E31" s="10" t="inlineStr">
-        <is>
-          <t>Bookmarks, drill-through, buttons, page links</t>
-        </is>
-      </c>
+      <c r="F31" s="51" t="n"/>
     </row>
     <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="51" t="n"/>
       <c r="B32" s="8" t="inlineStr">
         <is>
           <t>11</t>
@@ -1192,7 +1270,7 @@
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
-          <t>🎨 UI/UX Testing</t>
+          <t>🎨 S-11 UI-UX Testing</t>
         </is>
       </c>
       <c r="D32" s="8" t="inlineStr">
@@ -1205,8 +1283,10 @@
           <t>Layout, branding, fonts, colours, consistency</t>
         </is>
       </c>
+      <c r="F32" s="51" t="n"/>
     </row>
     <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="51" t="n"/>
       <c r="B33" s="10" t="inlineStr">
         <is>
           <t>12</t>
@@ -1214,7 +1294,7 @@
       </c>
       <c r="C33" s="10" t="inlineStr">
         <is>
-          <t>🔒 Security Testing</t>
+          <t>🔒 S-12 Security Testing</t>
         </is>
       </c>
       <c r="D33" s="10" t="inlineStr">
@@ -1227,8 +1307,10 @@
           <t>RLS, OLS, workspace permissions, sensitivity labels</t>
         </is>
       </c>
+      <c r="F33" s="51" t="n"/>
     </row>
     <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="51" t="n"/>
       <c r="B34" s="8" t="inlineStr">
         <is>
           <t>13</t>
@@ -1236,7 +1318,7 @@
       </c>
       <c r="C34" s="8" t="inlineStr">
         <is>
-          <t>🔄 Refresh Testing</t>
+          <t>🔄 S-13 Refresh Testing</t>
         </is>
       </c>
       <c r="D34" s="8" t="inlineStr">
@@ -1249,8 +1331,10 @@
           <t>Scheduled, incremental, manual refresh and alerts</t>
         </is>
       </c>
+      <c r="F34" s="51" t="n"/>
     </row>
     <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="51" t="n"/>
       <c r="B35" s="10" t="inlineStr">
         <is>
           <t>14</t>
@@ -1258,7 +1342,7 @@
       </c>
       <c r="C35" s="10" t="inlineStr">
         <is>
-          <t>⚡ Performance Testing</t>
+          <t>⚡ S-14 Performance Testing</t>
         </is>
       </c>
       <c r="D35" s="10" t="inlineStr">
@@ -1271,8 +1355,10 @@
           <t>Load times, DAX performance, concurrent users</t>
         </is>
       </c>
+      <c r="F35" s="51" t="n"/>
     </row>
     <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="51" t="n"/>
       <c r="B36" s="8" t="inlineStr">
         <is>
           <t>15</t>
@@ -1280,7 +1366,7 @@
       </c>
       <c r="C36" s="8" t="inlineStr">
         <is>
-          <t>♿ Accessibility Testing</t>
+          <t>♿ S-15 Accessibility Testing</t>
         </is>
       </c>
       <c r="D36" s="8" t="inlineStr">
@@ -1293,8 +1379,10 @@
           <t>Alt text, tab order, contrast, screen reader</t>
         </is>
       </c>
+      <c r="F36" s="51" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="51" t="n"/>
       <c r="B37" s="10" t="inlineStr">
         <is>
           <t>16</t>
@@ -1302,7 +1390,7 @@
       </c>
       <c r="C37" s="10" t="inlineStr">
         <is>
-          <t>📱 Mobile Layout</t>
+          <t>📱 S-16 Mobile Layout Testing</t>
         </is>
       </c>
       <c r="D37" s="10" t="inlineStr">
@@ -1315,8 +1403,10 @@
           <t>Mobile view, Power BI app, portrait/landscape</t>
         </is>
       </c>
+      <c r="F37" s="51" t="n"/>
     </row>
     <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="51" t="n"/>
       <c r="B38" s="8" t="inlineStr">
         <is>
           <t>17</t>
@@ -1324,7 +1414,7 @@
       </c>
       <c r="C38" s="8" t="inlineStr">
         <is>
-          <t>☁ Service Sanity</t>
+          <t>☁ S-17 Service Sanity Testing</t>
         </is>
       </c>
       <c r="D38" s="8" t="inlineStr">
@@ -1337,8 +1427,10 @@
           <t>Power BI Service deployment, workspace, sharing</t>
         </is>
       </c>
+      <c r="F38" s="51" t="n"/>
     </row>
     <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="51" t="n"/>
       <c r="B39" s="10" t="inlineStr">
         <is>
           <t>18</t>
@@ -1346,7 +1438,7 @@
       </c>
       <c r="C39" s="10" t="inlineStr">
         <is>
-          <t>📤 Export &amp; Subscription</t>
+          <t>📤 S-18 Export &amp; Subscription Testing</t>
         </is>
       </c>
       <c r="D39" s="10" t="inlineStr">
@@ -1359,8 +1451,10 @@
           <t>PDF, PPT, data export, email subscriptions</t>
         </is>
       </c>
+      <c r="F39" s="51" t="n"/>
     </row>
     <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="51" t="n"/>
       <c r="B40" s="8" t="inlineStr">
         <is>
           <t>19</t>
@@ -1368,7 +1462,7 @@
       </c>
       <c r="C40" s="8" t="inlineStr">
         <is>
-          <t>🔁 Regression Testing</t>
+          <t>🔁 S-19 Regression Testing</t>
         </is>
       </c>
       <c r="D40" s="8" t="inlineStr">
@@ -1381,8 +1475,10 @@
           <t>Re-test after changes, change impact matrix</t>
         </is>
       </c>
+      <c r="F40" s="51" t="n"/>
     </row>
     <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="51" t="n"/>
       <c r="B41" s="10" t="inlineStr">
         <is>
           <t>20</t>
@@ -1390,7 +1486,7 @@
       </c>
       <c r="C41" s="10" t="inlineStr">
         <is>
-          <t>✅ UAT Validation</t>
+          <t>✅ S-20 UAT Validation</t>
         </is>
       </c>
       <c r="D41" s="10" t="inlineStr">
@@ -1403,8 +1499,10 @@
           <t>Business sign-off, acceptance criteria, approvals</t>
         </is>
       </c>
+      <c r="F41" s="51" t="n"/>
     </row>
     <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="51" t="n"/>
       <c r="B42" s="8" t="inlineStr">
         <is>
           <t>21</t>
@@ -1412,7 +1510,7 @@
       </c>
       <c r="C42" s="8" t="inlineStr">
         <is>
-          <t>🚀 Deployment Validation</t>
+          <t>🚀 S-21 Deployment Validation</t>
         </is>
       </c>
       <c r="D42" s="8" t="inlineStr">
@@ -1422,11 +1520,13 @@
       </c>
       <c r="E42" s="8" t="inlineStr">
         <is>
-          <t>Pre/post deployment checks, smoke tests, rollback plan</t>
-        </is>
-      </c>
+          <t>Pre/post deployment checks, smoke tests, rollback</t>
+        </is>
+      </c>
+      <c r="F42" s="51" t="n"/>
     </row>
     <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="51" t="n"/>
       <c r="B43" s="10" t="inlineStr">
         <is>
           <t>—</t>
@@ -1447,8 +1547,10 @@
           <t>Defect tracking, severity, lifecycle</t>
         </is>
       </c>
+      <c r="F43" s="51" t="n"/>
     </row>
     <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="51" t="n"/>
       <c r="B44" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -1469,8 +1571,10 @@
           <t>Final sign-off summary and approvals</t>
         </is>
       </c>
+      <c r="F44" s="51" t="n"/>
     </row>
     <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="51" t="n"/>
       <c r="B45" s="10" t="inlineStr">
         <is>
           <t>—</t>
@@ -1488,12 +1592,131 @@
       </c>
       <c r="E45" s="10" t="inlineStr">
         <is>
-          <t>Quick check card for testers</t>
-        </is>
-      </c>
+          <t>Quick check card — all 21 categories</t>
+        </is>
+      </c>
+      <c r="F45" s="51" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="51" t="n"/>
+      <c r="B46" s="51" t="n"/>
+      <c r="C46" s="51" t="n"/>
+      <c r="D46" s="51" t="n"/>
+      <c r="E46" s="51" t="n"/>
+      <c r="F46" s="51" t="n"/>
+    </row>
+    <row r="47" ht="10" customHeight="1">
+      <c r="A47" s="51" t="n"/>
+      <c r="B47" s="51" t="n"/>
+      <c r="C47" s="51" t="n"/>
+      <c r="D47" s="51" t="n"/>
+      <c r="E47" s="51" t="n"/>
+      <c r="F47" s="51" t="n"/>
+    </row>
+    <row r="48" ht="28" customHeight="1">
+      <c r="A48" s="51" t="n"/>
+      <c r="B48" s="52" t="inlineStr">
+        <is>
+          <t>Testing Lifecycle Flow:  Requirements → Data Sources → Power Query → Data Validation → Data Model → DAX → Functional → Filters/Slicers → Navigation → Visuals → UI/UX → Security → Refresh → Performance → Accessibility → Mobile → Service → Export → Regression → UAT → Deployment</t>
+        </is>
+      </c>
+      <c r="F48" s="51" t="n"/>
+    </row>
+    <row r="49" ht="28" customHeight="1">
+      <c r="A49" s="51" t="n"/>
+      <c r="F49" s="51" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="51" t="n"/>
+      <c r="B50" s="51" t="n"/>
+      <c r="C50" s="51" t="n"/>
+      <c r="D50" s="51" t="n"/>
+      <c r="E50" s="51" t="n"/>
+      <c r="F50" s="51" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="51" t="n"/>
+      <c r="B51" s="51" t="n"/>
+      <c r="C51" s="51" t="n"/>
+      <c r="D51" s="51" t="n"/>
+      <c r="E51" s="51" t="n"/>
+      <c r="F51" s="51" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="51" t="n"/>
+      <c r="B52" s="51" t="n"/>
+      <c r="C52" s="51" t="n"/>
+      <c r="D52" s="51" t="n"/>
+      <c r="E52" s="51" t="n"/>
+      <c r="F52" s="51" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="51" t="n"/>
+      <c r="B53" s="51" t="n"/>
+      <c r="C53" s="51" t="n"/>
+      <c r="D53" s="51" t="n"/>
+      <c r="E53" s="51" t="n"/>
+      <c r="F53" s="51" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="51" t="n"/>
+      <c r="B54" s="51" t="n"/>
+      <c r="C54" s="51" t="n"/>
+      <c r="D54" s="51" t="n"/>
+      <c r="E54" s="51" t="n"/>
+      <c r="F54" s="51" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="51" t="n"/>
+      <c r="B55" s="51" t="n"/>
+      <c r="C55" s="51" t="n"/>
+      <c r="D55" s="51" t="n"/>
+      <c r="E55" s="51" t="n"/>
+      <c r="F55" s="51" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="51" t="n"/>
+      <c r="B56" s="51" t="n"/>
+      <c r="C56" s="51" t="n"/>
+      <c r="D56" s="51" t="n"/>
+      <c r="E56" s="51" t="n"/>
+      <c r="F56" s="51" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="51" t="n"/>
+      <c r="B57" s="51" t="n"/>
+      <c r="C57" s="51" t="n"/>
+      <c r="D57" s="51" t="n"/>
+      <c r="E57" s="51" t="n"/>
+      <c r="F57" s="51" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="51" t="n"/>
+      <c r="B58" s="51" t="n"/>
+      <c r="C58" s="51" t="n"/>
+      <c r="D58" s="51" t="n"/>
+      <c r="E58" s="51" t="n"/>
+      <c r="F58" s="51" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="51" t="n"/>
+      <c r="B59" s="51" t="n"/>
+      <c r="C59" s="51" t="n"/>
+      <c r="D59" s="51" t="n"/>
+      <c r="E59" s="51" t="n"/>
+      <c r="F59" s="51" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="51" t="n"/>
+      <c r="B60" s="51" t="n"/>
+      <c r="C60" s="51" t="n"/>
+      <c r="D60" s="51" t="n"/>
+      <c r="E60" s="51" t="n"/>
+      <c r="F60" s="51" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
+    <mergeCell ref="B48:E49"/>
     <mergeCell ref="B8:E9"/>
     <mergeCell ref="B2:E4"/>
     <mergeCell ref="B11:E12"/>
@@ -1505,6 +1728,589 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>🧭 S-10 NAVIGATION TESTING</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t>Test all bookmarks, drill-through pages, navigation buttons, and page-level linking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="8" customHeight="1"/>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>1. Bookmark Testing</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>Test ID</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>Validation Point</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="inlineStr">
+        <is>
+          <t>Steps / How to Test</t>
+        </is>
+      </c>
+      <c r="D5" s="15" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="F5" s="15" t="inlineStr">
+        <is>
+          <t>Pass / Fail</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>NT-01</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Bookmark captures correct visual state</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Create/activate bookmark; verify filters, sort, and visible visuals</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Correct state captured</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr"/>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>☐ Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>NT-02</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Bookmark navigation button triggers correctly</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>Click button linked to bookmark; verify state loads</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>Correct bookmark state applied</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr"/>
+      <c r="F7" s="19" t="inlineStr">
+        <is>
+          <t>☐ Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>NT-03</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Bookmark restores after page navigation</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Activate bookmark, navigate away, return; verify state</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>State restores on return</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr"/>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>☐ Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>NT-04</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Page-level vs report-level bookmark scope</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>Verify bookmark scope (page/report) matches design</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>Correct scope applied</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr"/>
+      <c r="F9" s="19" t="inlineStr">
+        <is>
+          <t>☐ Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>NT-05</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Bookmark resets filters correctly</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Activate reset bookmark; verify all filters cleared</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>Filters cleared on bookmark</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr"/>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>☐ Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="8" customHeight="1"/>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>2. Drill-Through Testing</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>Test ID</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="inlineStr">
+        <is>
+          <t>Validation Point</t>
+        </is>
+      </c>
+      <c r="C13" s="15" t="inlineStr">
+        <is>
+          <t>Steps / How to Test</t>
+        </is>
+      </c>
+      <c r="D13" s="15" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="F13" s="15" t="inlineStr">
+        <is>
+          <t>Pass / Fail</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>NT-06</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>Drill-through menu appears on right-click</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Right-click data point; verify drill-through pages listed</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Correct pages in context menu</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr"/>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>☐ Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>NT-07</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Drill-through carries correct filter context</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>Drill through from a data point; verify target page filtered</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>Target page shows correct context</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="inlineStr"/>
+      <c r="F15" s="19" t="inlineStr">
+        <is>
+          <t>☐ Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>NT-08</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Back button returns to source page</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>On drill-through page, click Back; verify return</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Returns to origin page and state</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr"/>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>☐ Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>NT-09</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>Drill-through restricted to authorised users</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>Test drill-through access by role</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>Unauthorised roles cannot access</t>
+        </is>
+      </c>
+      <c r="E17" s="10" t="inlineStr"/>
+      <c r="F17" s="19" t="inlineStr">
+        <is>
+          <t>☐ Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>NT-10</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>Cross-report drill-through works</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Drill-through to another report; verify context passed</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>Target report opens with correct filter</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr"/>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>☐ Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="8" customHeight="1"/>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>3. Button &amp; Page Navigation Testing</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>Test ID</t>
+        </is>
+      </c>
+      <c r="B21" s="15" t="inlineStr">
+        <is>
+          <t>Validation Point</t>
+        </is>
+      </c>
+      <c r="C21" s="15" t="inlineStr">
+        <is>
+          <t>Steps / How to Test</t>
+        </is>
+      </c>
+      <c r="D21" s="15" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="E21" s="15" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="F21" s="15" t="inlineStr">
+        <is>
+          <t>Pass / Fail</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>NT-11</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>Navigation button links to correct page</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Click each navigation button; verify destination</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>Correct page displayed</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr"/>
+      <c r="F22" s="18" t="inlineStr">
+        <is>
+          <t>☐ Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>NT-12</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>Conditional visibility of buttons works</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>Trigger visibility condition; verify button shows/hides</t>
+        </is>
+      </c>
+      <c r="D23" s="10" t="inlineStr">
+        <is>
+          <t>Correct visibility behaviour</t>
+        </is>
+      </c>
+      <c r="E23" s="10" t="inlineStr"/>
+      <c r="F23" s="19" t="inlineStr">
+        <is>
+          <t>☐ Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>NT-13</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>External URL buttons open correctly</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Click URL buttons; verify correct URL opens in new tab</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>Correct URL opened</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr"/>
+      <c r="F24" s="18" t="inlineStr">
+        <is>
+          <t>☐ Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>NT-14</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>Page tabs navigate correctly</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>Click each page tab; verify correct page loads</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="inlineStr">
+        <is>
+          <t>Correct page content shown</t>
+        </is>
+      </c>
+      <c r="E25" s="10" t="inlineStr"/>
+      <c r="F25" s="19" t="inlineStr">
+        <is>
+          <t>☐ Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>NT-15</t>
+        </is>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>Custom tooltip page appears on hover</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>Hover over visual; verify custom tooltip page loads</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>Tooltip content correct for data point</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr"/>
+      <c r="F26" s="18" t="inlineStr">
+        <is>
+          <t>☐ Pending</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A20:F20"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1524,14 +2330,14 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="12" t="inlineStr">
         <is>
-          <t>🔽 S-09 FILTER &amp; SLICER TESTING</t>
+          <t>👁 S-08 VISUAL VALIDATION</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>Test all filter panel types, slicer configurations, sync behaviour, and default filter states.</t>
+          <t>Validate chart types, visual formatting, tooltips, axis labels, totals, and conditional formatting.</t>
         </is>
       </c>
     </row>
@@ -1539,7 +2345,7 @@
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>1. Slicer Behaviour Test Cases</t>
+          <t>1. Visual Configuration Checklist</t>
         </is>
       </c>
     </row>
@@ -1556,17 +2362,17 @@
       </c>
       <c r="C5" s="15" t="inlineStr">
         <is>
-          <t>Steps / How to Test</t>
+          <t>What to Check</t>
         </is>
       </c>
       <c r="D5" s="15" t="inlineStr">
         <is>
-          <t>Expected Result</t>
+          <t>Issue Found?</t>
         </is>
       </c>
       <c r="E5" s="15" t="inlineStr">
         <is>
-          <t>Actual Result</t>
+          <t>Notes</t>
         </is>
       </c>
       <c r="F5" s="15" t="inlineStr">
@@ -1578,22 +2384,22 @@
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>FS-01</t>
+          <t>VV-01</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>Single-select slicer — correct value shown</t>
+          <t>Correct visual type used</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>Select one value; verify all visuals reflect that single value</t>
+          <t>Visual type is appropriate for the data being shown</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>All visuals filter correctly</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr"/>
@@ -1606,22 +2412,22 @@
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>FS-02</t>
+          <t>VV-02</t>
         </is>
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>Multi-select slicer — OR logic applied</t>
+          <t>Chart axis labels correct</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>Select multiple values; verify visuals show union</t>
+          <t>X and Y axis labels correctly named and formatted</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>OR logic applied correctly</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E7" s="10" t="inlineStr"/>
@@ -1634,22 +2440,22 @@
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>FS-03</t>
+          <t>VV-03</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>'Select All' selects all values</t>
+          <t>Legend labels and colours correct</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>Click Select All; verify full unfiltered data shown</t>
+          <t>Legend items labelled correctly, match colours used</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>All values selected, full data visible</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr"/>
@@ -1662,22 +2468,22 @@
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>FS-04</t>
+          <t>VV-04</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>'Deselect All' clears all selections</t>
+          <t>Data labels formatted correctly</t>
         </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>Click Deselect All; verify blank/empty state</t>
+          <t>Data labels show values with correct format/decimals</t>
         </is>
       </c>
       <c r="D9" s="10" t="inlineStr">
         <is>
-          <t>All visuals show blank or empty</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E9" s="10" t="inlineStr"/>
@@ -1690,22 +2496,22 @@
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>FS-05</t>
+          <t>VV-05</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Slicer search functionality</t>
+          <t>Default sort order correct</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>Type in slicer search box; verify filtered list</t>
+          <t>Sort is correct (e.g., descending value, ascending date)</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>Correct matching items returned</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr"/>
@@ -1718,22 +2524,22 @@
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>FS-06</t>
+          <t>VV-06</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>Date range slicer restricts correctly</t>
+          <t>Visual totals / subtotals correct</t>
         </is>
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>Set start and end dates; verify only that range shown</t>
+          <t>Matrix/table row and column totals are mathematically correct</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>Data within date range only</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E11" s="10" t="inlineStr"/>
@@ -1746,22 +2552,22 @@
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>FS-07</t>
+          <t>VV-07</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Between / before / after date slicer</t>
+          <t>Conditional formatting applied correctly</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>Test each date filter mode</t>
+          <t>Data bars, colour scales, icons apply per specification</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>Correct date filter applied</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr"/>
@@ -1774,22 +2580,22 @@
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>FS-08</t>
+          <t>VV-08</t>
         </is>
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>Slicer sync across pages</t>
+          <t>Custom tooltip content accurate</t>
         </is>
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>Apply slicer on Page 1; navigate to Page 2; verify sync</t>
+          <t>Tooltip shows correct fields for the hovered data point</t>
         </is>
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>Slicer value synced to Page 2</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E13" s="10" t="inlineStr"/>
@@ -1802,22 +2608,22 @@
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>FS-09</t>
+          <t>VV-09</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Default slicer value on report open</t>
+          <t>Map visual plots locations correctly</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Open report fresh; verify pre-set default filter value</t>
+          <t>Geographic locations resolve without misplotting</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>Default value applied on open</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr"/>
@@ -1830,22 +2636,22 @@
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>FS-10</t>
+          <t>VV-10</t>
         </is>
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>Clear filter on individual slicer</t>
+          <t>KPI trend direction logically correct</t>
         </is>
       </c>
       <c r="C15" s="10" t="inlineStr">
         <is>
-          <t>Click Clear icon; verify that slicer resets only</t>
+          <t>Up arrow = improvement, Down arrow = decline as defined</t>
         </is>
       </c>
       <c r="D15" s="10" t="inlineStr">
         <is>
-          <t>Slicer resets; others unchanged</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E15" s="10" t="inlineStr"/>
@@ -1858,22 +2664,22 @@
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>FS-11</t>
+          <t>VV-11</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Filter pane filters applied correctly</t>
+          <t>Card values update with slicer context</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>Use report/page/visual level filters in filter pane</t>
+          <t>Card values recalculate correctly when slicers applied</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>Correct scope of filter applied</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr"/>
@@ -1886,22 +2692,22 @@
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>FS-12</t>
+          <t>VV-12</t>
         </is>
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>Report-level filter restricts all pages</t>
+          <t>No truncated or overlapping labels</t>
         </is>
       </c>
       <c r="C17" s="10" t="inlineStr">
         <is>
-          <t>Set report-level filter; navigate all pages</t>
+          <t>All labels fully visible; no overlap with other elements</t>
         </is>
       </c>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t>All pages show filtered data</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E17" s="10" t="inlineStr"/>
@@ -1914,22 +2720,22 @@
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>FS-13</t>
+          <t>VV-13</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>Visual-level filter restricts single visual</t>
+          <t>Empty state / no-data message shown</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>Set visual filter; verify only that visual affected</t>
+          <t>Visuals display a meaningful message when no data exists</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>Only target visual filtered</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr"/>
@@ -1942,22 +2748,22 @@
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>FS-14</t>
+          <t>VV-14</t>
         </is>
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>Relative date filter (last N days/months)</t>
+          <t>Paginated report layout correct</t>
         </is>
       </c>
       <c r="C19" s="10" t="inlineStr">
         <is>
-          <t>Set relative date filter; verify date window rolls</t>
+          <t>Headers, footers, and page breaks render as designed</t>
         </is>
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>Rolling date filter correct</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E19" s="10" t="inlineStr"/>
@@ -1972,589 +2778,6 @@
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A4:F4"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F26"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="38" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
-        <is>
-          <t>🧭 S-10 NAVIGATION TESTING</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="13" t="inlineStr">
-        <is>
-          <t>Test all bookmarks, drill-through pages, navigation buttons, and page-level linking.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="8" customHeight="1"/>
-    <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="14" t="inlineStr">
-        <is>
-          <t>1. Bookmark Testing</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="15" t="inlineStr">
-        <is>
-          <t>Test ID</t>
-        </is>
-      </c>
-      <c r="B5" s="15" t="inlineStr">
-        <is>
-          <t>Validation Point</t>
-        </is>
-      </c>
-      <c r="C5" s="15" t="inlineStr">
-        <is>
-          <t>Steps / How to Test</t>
-        </is>
-      </c>
-      <c r="D5" s="15" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="E5" s="15" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="F5" s="15" t="inlineStr">
-        <is>
-          <t>Pass / Fail</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>NT-01</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>Bookmark captures correct visual state</t>
-        </is>
-      </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>Create/activate bookmark; verify filters, sort, and visible visuals</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>Correct state captured</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="inlineStr"/>
-      <c r="F6" s="18" t="inlineStr">
-        <is>
-          <t>☐ Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="10" t="inlineStr">
-        <is>
-          <t>NT-02</t>
-        </is>
-      </c>
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t>Bookmark navigation button triggers correctly</t>
-        </is>
-      </c>
-      <c r="C7" s="10" t="inlineStr">
-        <is>
-          <t>Click button linked to bookmark; verify state loads</t>
-        </is>
-      </c>
-      <c r="D7" s="10" t="inlineStr">
-        <is>
-          <t>Correct bookmark state applied</t>
-        </is>
-      </c>
-      <c r="E7" s="10" t="inlineStr"/>
-      <c r="F7" s="19" t="inlineStr">
-        <is>
-          <t>☐ Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>NT-03</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>Bookmark restores after page navigation</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>Activate bookmark, navigate away, return; verify state</t>
-        </is>
-      </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>State restores on return</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="inlineStr"/>
-      <c r="F8" s="18" t="inlineStr">
-        <is>
-          <t>☐ Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t>NT-04</t>
-        </is>
-      </c>
-      <c r="B9" s="10" t="inlineStr">
-        <is>
-          <t>Page-level vs report-level bookmark scope</t>
-        </is>
-      </c>
-      <c r="C9" s="10" t="inlineStr">
-        <is>
-          <t>Verify bookmark scope (page/report) matches design</t>
-        </is>
-      </c>
-      <c r="D9" s="10" t="inlineStr">
-        <is>
-          <t>Correct scope applied</t>
-        </is>
-      </c>
-      <c r="E9" s="10" t="inlineStr"/>
-      <c r="F9" s="19" t="inlineStr">
-        <is>
-          <t>☐ Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>NT-05</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>Bookmark resets filters correctly</t>
-        </is>
-      </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>Activate reset bookmark; verify all filters cleared</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>Filters cleared on bookmark</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="inlineStr"/>
-      <c r="F10" s="18" t="inlineStr">
-        <is>
-          <t>☐ Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="8" customHeight="1"/>
-    <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="14" t="inlineStr">
-        <is>
-          <t>2. Drill-Through Testing</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="15" t="inlineStr">
-        <is>
-          <t>Test ID</t>
-        </is>
-      </c>
-      <c r="B13" s="15" t="inlineStr">
-        <is>
-          <t>Validation Point</t>
-        </is>
-      </c>
-      <c r="C13" s="15" t="inlineStr">
-        <is>
-          <t>Steps / How to Test</t>
-        </is>
-      </c>
-      <c r="D13" s="15" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="E13" s="15" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="F13" s="15" t="inlineStr">
-        <is>
-          <t>Pass / Fail</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="8" t="inlineStr">
-        <is>
-          <t>NT-06</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>Drill-through menu appears on right-click</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>Right-click data point; verify drill-through pages listed</t>
-        </is>
-      </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>Correct pages in context menu</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="inlineStr"/>
-      <c r="F14" s="18" t="inlineStr">
-        <is>
-          <t>☐ Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="10" t="inlineStr">
-        <is>
-          <t>NT-07</t>
-        </is>
-      </c>
-      <c r="B15" s="10" t="inlineStr">
-        <is>
-          <t>Drill-through carries correct filter context</t>
-        </is>
-      </c>
-      <c r="C15" s="10" t="inlineStr">
-        <is>
-          <t>Drill through from a data point; verify target page filtered</t>
-        </is>
-      </c>
-      <c r="D15" s="10" t="inlineStr">
-        <is>
-          <t>Target page shows correct context</t>
-        </is>
-      </c>
-      <c r="E15" s="10" t="inlineStr"/>
-      <c r="F15" s="19" t="inlineStr">
-        <is>
-          <t>☐ Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="8" t="inlineStr">
-        <is>
-          <t>NT-08</t>
-        </is>
-      </c>
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>Back button returns to source page</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="inlineStr">
-        <is>
-          <t>On drill-through page, click Back; verify return</t>
-        </is>
-      </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>Returns to origin page and state</t>
-        </is>
-      </c>
-      <c r="E16" s="8" t="inlineStr"/>
-      <c r="F16" s="18" t="inlineStr">
-        <is>
-          <t>☐ Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="10" t="inlineStr">
-        <is>
-          <t>NT-09</t>
-        </is>
-      </c>
-      <c r="B17" s="10" t="inlineStr">
-        <is>
-          <t>Drill-through restricted to authorised users</t>
-        </is>
-      </c>
-      <c r="C17" s="10" t="inlineStr">
-        <is>
-          <t>Test drill-through access by role</t>
-        </is>
-      </c>
-      <c r="D17" s="10" t="inlineStr">
-        <is>
-          <t>Unauthorised roles cannot access</t>
-        </is>
-      </c>
-      <c r="E17" s="10" t="inlineStr"/>
-      <c r="F17" s="19" t="inlineStr">
-        <is>
-          <t>☐ Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="8" t="inlineStr">
-        <is>
-          <t>NT-10</t>
-        </is>
-      </c>
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>Cross-report drill-through works</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>Drill-through to another report; verify context passed</t>
-        </is>
-      </c>
-      <c r="D18" s="8" t="inlineStr">
-        <is>
-          <t>Target report opens with correct filter</t>
-        </is>
-      </c>
-      <c r="E18" s="8" t="inlineStr"/>
-      <c r="F18" s="18" t="inlineStr">
-        <is>
-          <t>☐ Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="8" customHeight="1"/>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="14" t="inlineStr">
-        <is>
-          <t>3. Button &amp; Page Navigation Testing</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="15" t="inlineStr">
-        <is>
-          <t>Test ID</t>
-        </is>
-      </c>
-      <c r="B21" s="15" t="inlineStr">
-        <is>
-          <t>Validation Point</t>
-        </is>
-      </c>
-      <c r="C21" s="15" t="inlineStr">
-        <is>
-          <t>Steps / How to Test</t>
-        </is>
-      </c>
-      <c r="D21" s="15" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="E21" s="15" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="F21" s="15" t="inlineStr">
-        <is>
-          <t>Pass / Fail</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="8" t="inlineStr">
-        <is>
-          <t>NT-11</t>
-        </is>
-      </c>
-      <c r="B22" s="8" t="inlineStr">
-        <is>
-          <t>Navigation button links to correct page</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>Click each navigation button; verify destination</t>
-        </is>
-      </c>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <t>Correct page displayed</t>
-        </is>
-      </c>
-      <c r="E22" s="8" t="inlineStr"/>
-      <c r="F22" s="18" t="inlineStr">
-        <is>
-          <t>☐ Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="10" t="inlineStr">
-        <is>
-          <t>NT-12</t>
-        </is>
-      </c>
-      <c r="B23" s="10" t="inlineStr">
-        <is>
-          <t>Conditional visibility of buttons works</t>
-        </is>
-      </c>
-      <c r="C23" s="10" t="inlineStr">
-        <is>
-          <t>Trigger visibility condition; verify button shows/hides</t>
-        </is>
-      </c>
-      <c r="D23" s="10" t="inlineStr">
-        <is>
-          <t>Correct visibility behaviour</t>
-        </is>
-      </c>
-      <c r="E23" s="10" t="inlineStr"/>
-      <c r="F23" s="19" t="inlineStr">
-        <is>
-          <t>☐ Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="8" t="inlineStr">
-        <is>
-          <t>NT-13</t>
-        </is>
-      </c>
-      <c r="B24" s="8" t="inlineStr">
-        <is>
-          <t>External URL buttons open correctly</t>
-        </is>
-      </c>
-      <c r="C24" s="8" t="inlineStr">
-        <is>
-          <t>Click URL buttons; verify correct URL opens in new tab</t>
-        </is>
-      </c>
-      <c r="D24" s="8" t="inlineStr">
-        <is>
-          <t>Correct URL opened</t>
-        </is>
-      </c>
-      <c r="E24" s="8" t="inlineStr"/>
-      <c r="F24" s="18" t="inlineStr">
-        <is>
-          <t>☐ Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="10" t="inlineStr">
-        <is>
-          <t>NT-14</t>
-        </is>
-      </c>
-      <c r="B25" s="10" t="inlineStr">
-        <is>
-          <t>Page tabs navigate correctly</t>
-        </is>
-      </c>
-      <c r="C25" s="10" t="inlineStr">
-        <is>
-          <t>Click each page tab; verify correct page loads</t>
-        </is>
-      </c>
-      <c r="D25" s="10" t="inlineStr">
-        <is>
-          <t>Correct page content shown</t>
-        </is>
-      </c>
-      <c r="E25" s="10" t="inlineStr"/>
-      <c r="F25" s="19" t="inlineStr">
-        <is>
-          <t>☐ Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="8" t="inlineStr">
-        <is>
-          <t>NT-15</t>
-        </is>
-      </c>
-      <c r="B26" s="8" t="inlineStr">
-        <is>
-          <t>Custom tooltip page appears on hover</t>
-        </is>
-      </c>
-      <c r="C26" s="8" t="inlineStr">
-        <is>
-          <t>Hover over visual; verify custom tooltip page loads</t>
-        </is>
-      </c>
-      <c r="D26" s="8" t="inlineStr">
-        <is>
-          <t>Tooltip content correct for data point</t>
-        </is>
-      </c>
-      <c r="E26" s="8" t="inlineStr"/>
-      <c r="F26" s="18" t="inlineStr">
-        <is>
-          <t>☐ Pending</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A20:F20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4942,10 +5165,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A15:G15"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A4:G4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5886,9 +6109,9 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A17:F17"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A17:F17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6873,9 +7096,9 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A17:F17"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A17:F17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7299,9 +7522,9 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A17:F17"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A17:F17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7500,6 +7723,11 @@
           <t>DAX measures or calculated columns modified</t>
         </is>
       </c>
+      <c r="C19" s="53" t="n"/>
+      <c r="D19" s="53" t="n"/>
+      <c r="E19" s="53" t="n"/>
+      <c r="F19" s="53" t="n"/>
+      <c r="G19" s="54" t="n"/>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="22" t="inlineStr">
@@ -7512,6 +7740,11 @@
           <t>Power Query transformation steps changed</t>
         </is>
       </c>
+      <c r="C20" s="53" t="n"/>
+      <c r="D20" s="53" t="n"/>
+      <c r="E20" s="53" t="n"/>
+      <c r="F20" s="53" t="n"/>
+      <c r="G20" s="54" t="n"/>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="20" t="inlineStr">
@@ -7524,6 +7757,11 @@
           <t>Data source schema changed (columns added/renamed/removed)</t>
         </is>
       </c>
+      <c r="C21" s="53" t="n"/>
+      <c r="D21" s="53" t="n"/>
+      <c r="E21" s="53" t="n"/>
+      <c r="F21" s="53" t="n"/>
+      <c r="G21" s="54" t="n"/>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="22" t="inlineStr">
@@ -7536,6 +7774,11 @@
           <t>New data source added or existing source replaced</t>
         </is>
       </c>
+      <c r="C22" s="53" t="n"/>
+      <c r="D22" s="53" t="n"/>
+      <c r="E22" s="53" t="n"/>
+      <c r="F22" s="53" t="n"/>
+      <c r="G22" s="54" t="n"/>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="20" t="inlineStr">
@@ -7548,6 +7791,11 @@
           <t>Report visuals added, removed, or restructured</t>
         </is>
       </c>
+      <c r="C23" s="53" t="n"/>
+      <c r="D23" s="53" t="n"/>
+      <c r="E23" s="53" t="n"/>
+      <c r="F23" s="53" t="n"/>
+      <c r="G23" s="54" t="n"/>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="22" t="inlineStr">
@@ -7560,6 +7808,11 @@
           <t>RLS or OLS roles created, modified, or removed</t>
         </is>
       </c>
+      <c r="C24" s="53" t="n"/>
+      <c r="D24" s="53" t="n"/>
+      <c r="E24" s="53" t="n"/>
+      <c r="F24" s="53" t="n"/>
+      <c r="G24" s="54" t="n"/>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="20" t="inlineStr">
@@ -7572,6 +7825,11 @@
           <t>Power BI Desktop or Service platform version updated</t>
         </is>
       </c>
+      <c r="C25" s="53" t="n"/>
+      <c r="D25" s="53" t="n"/>
+      <c r="E25" s="53" t="n"/>
+      <c r="F25" s="53" t="n"/>
+      <c r="G25" s="54" t="n"/>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="22" t="inlineStr">
@@ -7584,6 +7842,11 @@
           <t>Data model relationships changed</t>
         </is>
       </c>
+      <c r="C26" s="53" t="n"/>
+      <c r="D26" s="53" t="n"/>
+      <c r="E26" s="53" t="n"/>
+      <c r="F26" s="53" t="n"/>
+      <c r="G26" s="54" t="n"/>
     </row>
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="20" t="inlineStr">
@@ -7596,6 +7859,11 @@
           <t>Calculated tables added or modified</t>
         </is>
       </c>
+      <c r="C27" s="53" t="n"/>
+      <c r="D27" s="53" t="n"/>
+      <c r="E27" s="53" t="n"/>
+      <c r="F27" s="53" t="n"/>
+      <c r="G27" s="54" t="n"/>
     </row>
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="22" t="inlineStr">
@@ -7608,6 +7876,11 @@
           <t>Report theme or branding updated</t>
         </is>
       </c>
+      <c r="C28" s="53" t="n"/>
+      <c r="D28" s="53" t="n"/>
+      <c r="E28" s="53" t="n"/>
+      <c r="F28" s="53" t="n"/>
+      <c r="G28" s="54" t="n"/>
     </row>
     <row r="29" ht="8" customHeight="1"/>
     <row r="30" ht="22" customHeight="1">
@@ -8336,6 +8609,11 @@
           <t>All Critical (P1) and High (P2) defects resolved and re-tested</t>
         </is>
       </c>
+      <c r="C40" s="53" t="n"/>
+      <c r="D40" s="53" t="n"/>
+      <c r="E40" s="53" t="n"/>
+      <c r="F40" s="53" t="n"/>
+      <c r="G40" s="54" t="n"/>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="A41" s="22" t="inlineStr">
@@ -8348,6 +8626,11 @@
           <t>No open defects exceed the agreed severity threshold</t>
         </is>
       </c>
+      <c r="C41" s="53" t="n"/>
+      <c r="D41" s="53" t="n"/>
+      <c r="E41" s="53" t="n"/>
+      <c r="F41" s="53" t="n"/>
+      <c r="G41" s="54" t="n"/>
     </row>
     <row r="42" ht="20" customHeight="1">
       <c r="A42" s="20" t="inlineStr">
@@ -8360,6 +8643,11 @@
           <t>At least 90% of UAT test cases have passed</t>
         </is>
       </c>
+      <c r="C42" s="53" t="n"/>
+      <c r="D42" s="53" t="n"/>
+      <c r="E42" s="53" t="n"/>
+      <c r="F42" s="53" t="n"/>
+      <c r="G42" s="54" t="n"/>
     </row>
     <row r="43" ht="20" customHeight="1">
       <c r="A43" s="22" t="inlineStr">
@@ -8372,6 +8660,11 @@
           <t>Data reconciliation confirms accuracy within agreed tolerance (±0.01%)</t>
         </is>
       </c>
+      <c r="C43" s="53" t="n"/>
+      <c r="D43" s="53" t="n"/>
+      <c r="E43" s="53" t="n"/>
+      <c r="F43" s="53" t="n"/>
+      <c r="G43" s="54" t="n"/>
     </row>
     <row r="44" ht="20" customHeight="1">
       <c r="A44" s="20" t="inlineStr">
@@ -8384,6 +8677,11 @@
           <t>Performance meets agreed load time thresholds</t>
         </is>
       </c>
+      <c r="C44" s="53" t="n"/>
+      <c r="D44" s="53" t="n"/>
+      <c r="E44" s="53" t="n"/>
+      <c r="F44" s="53" t="n"/>
+      <c r="G44" s="54" t="n"/>
     </row>
     <row r="45" ht="20" customHeight="1">
       <c r="A45" s="22" t="inlineStr">
@@ -8396,6 +8694,11 @@
           <t>RLS tested and confirmed for all roles</t>
         </is>
       </c>
+      <c r="C45" s="53" t="n"/>
+      <c r="D45" s="53" t="n"/>
+      <c r="E45" s="53" t="n"/>
+      <c r="F45" s="53" t="n"/>
+      <c r="G45" s="54" t="n"/>
     </row>
     <row r="46" ht="20" customHeight="1">
       <c r="A46" s="20" t="inlineStr">
@@ -8408,6 +8711,11 @@
           <t>Business Owner has reviewed and approved all report pages</t>
         </is>
       </c>
+      <c r="C46" s="53" t="n"/>
+      <c r="D46" s="53" t="n"/>
+      <c r="E46" s="53" t="n"/>
+      <c r="F46" s="53" t="n"/>
+      <c r="G46" s="54" t="n"/>
     </row>
     <row r="47" ht="20" customHeight="1">
       <c r="A47" s="22" t="inlineStr">
@@ -8420,6 +8728,11 @@
           <t>Formal written sign-off obtained from Business Owner</t>
         </is>
       </c>
+      <c r="C47" s="53" t="n"/>
+      <c r="D47" s="53" t="n"/>
+      <c r="E47" s="53" t="n"/>
+      <c r="F47" s="53" t="n"/>
+      <c r="G47" s="54" t="n"/>
     </row>
     <row r="48" ht="8" customHeight="1"/>
     <row r="49" ht="22" customHeight="1">
@@ -9402,6 +9715,11 @@
           <t>Complete the rollback plan BEFORE deploying. If smoke tests fail, execute rollback immediately.</t>
         </is>
       </c>
+      <c r="B40" s="53" t="n"/>
+      <c r="C40" s="53" t="n"/>
+      <c r="D40" s="53" t="n"/>
+      <c r="E40" s="53" t="n"/>
+      <c r="F40" s="54" t="n"/>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="A41" s="15" t="inlineStr">
@@ -9751,6 +10069,7 @@
           <t>Unusable / materially wrong data</t>
         </is>
       </c>
+      <c r="C5" s="54" t="n"/>
       <c r="D5" s="33" t="inlineStr">
         <is>
           <t>P2 – High</t>
@@ -9761,6 +10080,7 @@
           <t>Key functionality broken</t>
         </is>
       </c>
+      <c r="F5" s="54" t="n"/>
       <c r="G5" s="34" t="inlineStr">
         <is>
           <t>P3 – Medium</t>
@@ -9771,6 +10091,7 @@
           <t>Non-critical issue</t>
         </is>
       </c>
+      <c r="I5" s="54" t="n"/>
       <c r="J5" s="35" t="inlineStr">
         <is>
           <t>P4 – Low</t>
@@ -9781,6 +10102,7 @@
           <t>Cosmetic / minor</t>
         </is>
       </c>
+      <c r="L5" s="54" t="n"/>
     </row>
     <row r="6" ht="8" customHeight="1"/>
     <row r="7" ht="30" customHeight="1">
@@ -10648,7 +10970,7 @@
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="23" t="inlineStr">
         <is>
-          <t>08  Visual Validation</t>
+          <t>08  Filter &amp; Slicer Testing</t>
         </is>
       </c>
       <c r="B13" s="39" t="inlineStr">
@@ -10668,7 +10990,7 @@
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="21" t="inlineStr">
         <is>
-          <t>09  Filter &amp; Slicer Testing</t>
+          <t>09  Navigation Testing</t>
         </is>
       </c>
       <c r="B14" s="38" t="inlineStr">
@@ -10688,7 +11010,7 @@
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="23" t="inlineStr">
         <is>
-          <t>10  Navigation Testing</t>
+          <t>10  Visual Validation</t>
         </is>
       </c>
       <c r="B15" s="39" t="inlineStr">
@@ -11075,11 +11397,15 @@
           <t>✅  GO — Approved for deployment to production</t>
         </is>
       </c>
+      <c r="B40" s="53" t="n"/>
+      <c r="C40" s="53" t="n"/>
+      <c r="D40" s="54" t="n"/>
       <c r="E40" s="43" t="inlineStr">
         <is>
           <t>☐  Select</t>
         </is>
       </c>
+      <c r="F40" s="54" t="n"/>
     </row>
     <row r="41" ht="26" customHeight="1">
       <c r="A41" s="44" t="inlineStr">
@@ -11087,18 +11413,22 @@
           <t>🚫  NO-GO — Further testing / defect resolution required</t>
         </is>
       </c>
+      <c r="B41" s="53" t="n"/>
+      <c r="C41" s="53" t="n"/>
+      <c r="D41" s="54" t="n"/>
       <c r="E41" s="43" t="inlineStr">
         <is>
           <t>☐  Select</t>
         </is>
       </c>
+      <c r="F41" s="54" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A40:D40"/>
+    <mergeCell ref="E41:F41"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="E41:F41"/>
     <mergeCell ref="E40:F40"/>
     <mergeCell ref="A41:D41"/>
     <mergeCell ref="A4:F4"/>
@@ -15245,14 +15575,14 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="12" t="inlineStr">
         <is>
-          <t>👁 S-08 VISUAL VALIDATION</t>
+          <t>🔽 S-09 FILTER &amp; SLICER TESTING</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>Validate chart types, visual formatting, tooltips, axis labels, totals, and conditional formatting.</t>
+          <t>Test all filter panel types, slicer configurations, sync behaviour, and default filter states.</t>
         </is>
       </c>
     </row>
@@ -15260,7 +15590,7 @@
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>1. Visual Configuration Checklist</t>
+          <t>1. Slicer Behaviour Test Cases</t>
         </is>
       </c>
     </row>
@@ -15277,17 +15607,17 @@
       </c>
       <c r="C5" s="15" t="inlineStr">
         <is>
-          <t>What to Check</t>
+          <t>Steps / How to Test</t>
         </is>
       </c>
       <c r="D5" s="15" t="inlineStr">
         <is>
-          <t>Issue Found?</t>
+          <t>Expected Result</t>
         </is>
       </c>
       <c r="E5" s="15" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>Actual Result</t>
         </is>
       </c>
       <c r="F5" s="15" t="inlineStr">
@@ -15299,22 +15629,22 @@
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>VV-01</t>
+          <t>FS-01</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>Correct visual type used</t>
+          <t>Single-select slicer — correct value shown</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>Visual type is appropriate for the data being shown</t>
+          <t>Select one value; verify all visuals reflect that single value</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>All visuals filter correctly</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr"/>
@@ -15327,22 +15657,22 @@
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>VV-02</t>
+          <t>FS-02</t>
         </is>
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>Chart axis labels correct</t>
+          <t>Multi-select slicer — OR logic applied</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>X and Y axis labels correctly named and formatted</t>
+          <t>Select multiple values; verify visuals show union</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>OR logic applied correctly</t>
         </is>
       </c>
       <c r="E7" s="10" t="inlineStr"/>
@@ -15355,22 +15685,22 @@
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>VV-03</t>
+          <t>FS-03</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Legend labels and colours correct</t>
+          <t>'Select All' selects all values</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>Legend items labelled correctly, match colours used</t>
+          <t>Click Select All; verify full unfiltered data shown</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>All values selected, full data visible</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr"/>
@@ -15383,22 +15713,22 @@
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>VV-04</t>
+          <t>FS-04</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>Data labels formatted correctly</t>
+          <t>'Deselect All' clears all selections</t>
         </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>Data labels show values with correct format/decimals</t>
+          <t>Click Deselect All; verify blank/empty state</t>
         </is>
       </c>
       <c r="D9" s="10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>All visuals show blank or empty</t>
         </is>
       </c>
       <c r="E9" s="10" t="inlineStr"/>
@@ -15411,22 +15741,22 @@
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>VV-05</t>
+          <t>FS-05</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Default sort order correct</t>
+          <t>Slicer search functionality</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>Sort is correct (e.g., descending value, ascending date)</t>
+          <t>Type in slicer search box; verify filtered list</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Correct matching items returned</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr"/>
@@ -15439,22 +15769,22 @@
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>VV-06</t>
+          <t>FS-06</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>Visual totals / subtotals correct</t>
+          <t>Date range slicer restricts correctly</t>
         </is>
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>Matrix/table row and column totals are mathematically correct</t>
+          <t>Set start and end dates; verify only that range shown</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Data within date range only</t>
         </is>
       </c>
       <c r="E11" s="10" t="inlineStr"/>
@@ -15467,22 +15797,22 @@
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>VV-07</t>
+          <t>FS-07</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Conditional formatting applied correctly</t>
+          <t>Between / before / after date slicer</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>Data bars, colour scales, icons apply per specification</t>
+          <t>Test each date filter mode</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Correct date filter applied</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr"/>
@@ -15495,22 +15825,22 @@
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>VV-08</t>
+          <t>FS-08</t>
         </is>
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>Custom tooltip content accurate</t>
+          <t>Slicer sync across pages</t>
         </is>
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>Tooltip shows correct fields for the hovered data point</t>
+          <t>Apply slicer on Page 1; navigate to Page 2; verify sync</t>
         </is>
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Slicer value synced to Page 2</t>
         </is>
       </c>
       <c r="E13" s="10" t="inlineStr"/>
@@ -15523,22 +15853,22 @@
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>VV-09</t>
+          <t>FS-09</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Map visual plots locations correctly</t>
+          <t>Default slicer value on report open</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Geographic locations resolve without misplotting</t>
+          <t>Open report fresh; verify pre-set default filter value</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Default value applied on open</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr"/>
@@ -15551,22 +15881,22 @@
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>VV-10</t>
+          <t>FS-10</t>
         </is>
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>KPI trend direction logically correct</t>
+          <t>Clear filter on individual slicer</t>
         </is>
       </c>
       <c r="C15" s="10" t="inlineStr">
         <is>
-          <t>Up arrow = improvement, Down arrow = decline as defined</t>
+          <t>Click Clear icon; verify that slicer resets only</t>
         </is>
       </c>
       <c r="D15" s="10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Slicer resets; others unchanged</t>
         </is>
       </c>
       <c r="E15" s="10" t="inlineStr"/>
@@ -15579,22 +15909,22 @@
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>VV-11</t>
+          <t>FS-11</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Card values update with slicer context</t>
+          <t>Filter pane filters applied correctly</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>Card values recalculate correctly when slicers applied</t>
+          <t>Use report/page/visual level filters in filter pane</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Correct scope of filter applied</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr"/>
@@ -15607,22 +15937,22 @@
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>VV-12</t>
+          <t>FS-12</t>
         </is>
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>No truncated or overlapping labels</t>
+          <t>Report-level filter restricts all pages</t>
         </is>
       </c>
       <c r="C17" s="10" t="inlineStr">
         <is>
-          <t>All labels fully visible; no overlap with other elements</t>
+          <t>Set report-level filter; navigate all pages</t>
         </is>
       </c>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>All pages show filtered data</t>
         </is>
       </c>
       <c r="E17" s="10" t="inlineStr"/>
@@ -15635,22 +15965,22 @@
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>VV-13</t>
+          <t>FS-13</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>Empty state / no-data message shown</t>
+          <t>Visual-level filter restricts single visual</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>Visuals display a meaningful message when no data exists</t>
+          <t>Set visual filter; verify only that visual affected</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Only target visual filtered</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr"/>
@@ -15663,22 +15993,22 @@
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>VV-14</t>
+          <t>FS-14</t>
         </is>
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>Paginated report layout correct</t>
+          <t>Relative date filter (last N days/months)</t>
         </is>
       </c>
       <c r="C19" s="10" t="inlineStr">
         <is>
-          <t>Headers, footers, and page breaks render as designed</t>
+          <t>Set relative date filter; verify date window rolls</t>
         </is>
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Rolling date filter correct</t>
         </is>
       </c>
       <c r="E19" s="10" t="inlineStr"/>

</xml_diff>